<commit_message>
Remove duplicate report files and update error processing
Deleted duplicate Excel report files from data-analysis-python subdirectories and updated several reports in the main EMPRESAS directory. Also removed redundant data_path assignment in 2-processamento_erros.py to streamline file loading.
</commit_message>
<xml_diff>
--- a/Integration-Quality/EMPRESAS/Relatorio - INOVENTS.xlsx
+++ b/Integration-Quality/EMPRESAS/Relatorio - INOVENTS.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ64"/>
+  <dimension ref="A1:AQ66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,10 +695,10 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>22649878</v>
+        <v>22679559</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>23459408</v>
+        <v>23484064</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
@@ -706,24 +706,24 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>45868.40864583333</v>
+        <v>45873.65900462963</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>45868.41383101852</v>
+        <v>45873.67644675926</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>EGHULO</t>
+          <t>B3NZNT</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -733,24 +733,26 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>AMANDA MAYARA HENRIQUE DE OLIVEIRA</t>
+          <t>BUENO BARBOSA/RENATA</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Jaqueline Rodrigues Teixeira</t>
+          <t>Danny Junqueira Martins</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Jaqueline Rodrigues Teixeira</t>
+          <t>Danny Junqueira Martins</t>
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>45867</v>
-      </c>
-      <c r="N2" s="5" t="n">
-        <v>4801518571</v>
+        <v>45873.65833333333</v>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
@@ -784,46 +786,48 @@
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>Grupo Diageo</t>
+          <t>Grupo Jti</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>Diageo Brasil</t>
+          <t>Jti Distribuidora - Sao Paulo - Vila Nova Conceicao</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
         <is>
-          <t>Cliente FEE no POS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="Y2" s="5" t="n">
-        <v>2243394807</v>
+        <v>2971556787</v>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>
       </c>
-      <c r="AA2" s="5" t="n">
-        <v>167526</v>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>ID152723</t>
+        </is>
       </c>
       <c r="AB2" s="5" t="n">
-        <v>1542.36</v>
+        <v>6420.23</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>77.64</v>
+        <v>464.43</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE2" s="5" t="n">
-        <v>154.23</v>
+        <v>0</v>
       </c>
       <c r="AF2" s="5" t="n">
         <v>0</v>
@@ -832,16 +836,16 @@
         <v>0</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>192.85</v>
+        <v>655.21</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
-          <t>Reserva importada via planilha. Solicitação: |PC:</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AJ2" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2243394807 já sendo utilizado para este fornecedor.</t>
+          <t>Verificação de bilhetes: Bilhete 2971556787 já sendo utilizado para este fornecedor.</t>
         </is>
       </c>
       <c r="AK2" s="5" t="inlineStr">
@@ -882,10 +886,10 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>22649878</v>
+        <v>22679559</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>23459409</v>
+        <v>23484078</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -893,24 +897,24 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>45868.40864583333</v>
+        <v>45873.65900462963</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>45868.41383101852</v>
+        <v>45873.67644675926</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>EGHULO</t>
+          <t>B3NZNT</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -920,24 +924,26 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>MARIA LUIZA PEREIRA LIRA</t>
+          <t>SIMOES BARBOSA/FRANCISCO</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Jaqueline Rodrigues Teixeira</t>
+          <t>Danny Junqueira Martins</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Jaqueline Rodrigues Teixeira</t>
+          <t>Danny Junqueira Martins</t>
         </is>
       </c>
       <c r="M3" s="6" t="n">
-        <v>45867</v>
-      </c>
-      <c r="N3" s="5" t="n">
-        <v>4801518571</v>
+        <v>45873.65833333333</v>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
@@ -971,46 +977,48 @@
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>Grupo Diageo</t>
+          <t>Grupo Jti</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>Diageo Brasil</t>
+          <t>Jti Distribuidora - Sao Paulo - Vila Nova Conceicao</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
         <is>
-          <t>Cliente FEE no POS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="X3" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>2243394807</v>
+        <v>2971556785</v>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>
       </c>
-      <c r="AA3" s="5" t="n">
-        <v>167526</v>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>ID152723</t>
+        </is>
       </c>
       <c r="AB3" s="5" t="n">
-        <v>1542.36</v>
+        <v>6420.23</v>
       </c>
       <c r="AC3" s="5" t="n">
-        <v>77.64</v>
+        <v>464.43</v>
       </c>
       <c r="AD3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE3" s="5" t="n">
-        <v>154.23</v>
+        <v>0</v>
       </c>
       <c r="AF3" s="5" t="n">
         <v>0</v>
@@ -1019,16 +1027,16 @@
         <v>0</v>
       </c>
       <c r="AH3" s="5" t="n">
-        <v>192.85</v>
+        <v>655.21</v>
       </c>
       <c r="AI3" s="5" t="inlineStr">
         <is>
-          <t>Reserva importada via planilha. Solicitação: |PC:</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AJ3" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2243394807 já sendo utilizado para este fornecedor.</t>
+          <t>Verificação de bilhetes: Bilhete 2971556787 já sendo utilizado para este fornecedor.</t>
         </is>
       </c>
       <c r="AK3" s="5" t="inlineStr">
@@ -1072,11 +1080,11 @@
         <v>22649878</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>23459410</v>
+        <v>23459408</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ACC03</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D4" s="6" t="n">
@@ -1087,12 +1095,12 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
@@ -1107,7 +1115,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>EVERTON NUNES DA SILVA</t>
+          <t>AMANDA MAYARA HENRIQUE DE OLIVEIRA</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1256,35 +1264,35 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>22649882</v>
+        <v>22649878</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>23459418</v>
+        <v>23459409</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>ACC01</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>45868.40885416666</v>
+        <v>45868.40864583333</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45868.41383101852</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>HNMBIK</t>
+          <t>EGHULO</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -1294,7 +1302,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>BARBARA MAGALHAES</t>
+          <t>MARIA LUIZA PEREIRA LIRA</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -1364,7 +1372,7 @@
         </is>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>2243398439</v>
+        <v>2243394807</v>
       </c>
       <c r="Z5" s="5" t="inlineStr">
         <is>
@@ -1375,16 +1383,16 @@
         <v>167526</v>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>683.05</v>
+        <v>1542.36</v>
       </c>
       <c r="AC5" s="5" t="n">
-        <v>31.44</v>
+        <v>77.64</v>
       </c>
       <c r="AD5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE5" s="5" t="n">
-        <v>68.25</v>
+        <v>154.23</v>
       </c>
       <c r="AF5" s="5" t="n">
         <v>0</v>
@@ -1393,7 +1401,7 @@
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="n">
-        <v>86.09999999999999</v>
+        <v>192.85</v>
       </c>
       <c r="AI5" s="5" t="inlineStr">
         <is>
@@ -1402,7 +1410,7 @@
       </c>
       <c r="AJ5" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2243398493 já sendo utilizado para este fornecedor.</t>
+          <t>Verificação de bilhetes: Bilhete 2243394807 já sendo utilizado para este fornecedor.</t>
         </is>
       </c>
       <c r="AK5" s="5" t="inlineStr">
@@ -1443,35 +1451,35 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>22649882</v>
+        <v>22649878</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>23459419</v>
+        <v>23459410</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC03</t>
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>45868.40885416666</v>
+        <v>45868.40864583333</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45868.41383101852</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>HNMBIK</t>
+          <t>EGHULO</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -1481,7 +1489,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>JAMYLE PINHEIRO FACANHA CAVALCANTE</t>
+          <t>EVERTON NUNES DA SILVA</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -1551,7 +1559,7 @@
         </is>
       </c>
       <c r="Y6" s="5" t="n">
-        <v>2243398440</v>
+        <v>2243394807</v>
       </c>
       <c r="Z6" s="5" t="inlineStr">
         <is>
@@ -1562,16 +1570,16 @@
         <v>167526</v>
       </c>
       <c r="AB6" s="5" t="n">
-        <v>683.05</v>
+        <v>1542.36</v>
       </c>
       <c r="AC6" s="5" t="n">
-        <v>31.44</v>
+        <v>77.64</v>
       </c>
       <c r="AD6" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE6" s="5" t="n">
-        <v>68.25</v>
+        <v>154.23</v>
       </c>
       <c r="AF6" s="5" t="n">
         <v>0</v>
@@ -1580,7 +1588,7 @@
         <v>0</v>
       </c>
       <c r="AH6" s="5" t="n">
-        <v>86.09999999999999</v>
+        <v>192.85</v>
       </c>
       <c r="AI6" s="5" t="inlineStr">
         <is>
@@ -1589,7 +1597,7 @@
       </c>
       <c r="AJ6" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2243398493 já sendo utilizado para este fornecedor.</t>
+          <t>Verificação de bilhetes: Bilhete 2243394807 já sendo utilizado para este fornecedor.</t>
         </is>
       </c>
       <c r="AK6" s="5" t="inlineStr">
@@ -1633,11 +1641,11 @@
         <v>22649882</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>23459420</v>
+        <v>23459418</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>ACC03</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
@@ -1648,12 +1656,12 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1668,7 +1676,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>CHRISTIANE GURGEL DO AMARAL CHAVES</t>
+          <t>BARBARA MAGALHAES</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1738,7 +1746,7 @@
         </is>
       </c>
       <c r="Y7" s="5" t="n">
-        <v>2243398441</v>
+        <v>2243398439</v>
       </c>
       <c r="Z7" s="5" t="inlineStr">
         <is>
@@ -1820,11 +1828,11 @@
         <v>22649882</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>23459421</v>
+        <v>23459419</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ACC04</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D8" s="6" t="n">
@@ -1835,12 +1843,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1855,7 +1863,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>HELEN LIDIA MENDES</t>
+          <t>JAMYLE PINHEIRO FACANHA CAVALCANTE</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1925,7 +1933,7 @@
         </is>
       </c>
       <c r="Y8" s="5" t="n">
-        <v>2243398442</v>
+        <v>2243398440</v>
       </c>
       <c r="Z8" s="5" t="inlineStr">
         <is>
@@ -2007,11 +2015,11 @@
         <v>22649882</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>23459422</v>
+        <v>23459420</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>ACC05</t>
+          <t>ACC03</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
@@ -2022,12 +2030,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -2042,7 +2050,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>DAMARIS RAQUELINA MALAQUIAS SARAIVA</t>
+          <t>CHRISTIANE GURGEL DO AMARAL CHAVES</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -2112,7 +2120,7 @@
         </is>
       </c>
       <c r="Y9" s="5" t="n">
-        <v>2243398443</v>
+        <v>2243398441</v>
       </c>
       <c r="Z9" s="5" t="inlineStr">
         <is>
@@ -2194,11 +2202,11 @@
         <v>22649882</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>23459423</v>
+        <v>23459421</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ACC06</t>
+          <t>ACC04</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
@@ -2209,12 +2217,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -2229,7 +2237,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>ANTONIA LETICIA DE SOUZA</t>
+          <t>HELEN LIDIA MENDES</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -2299,7 +2307,7 @@
         </is>
       </c>
       <c r="Y10" s="5" t="n">
-        <v>2243398444</v>
+        <v>2243398442</v>
       </c>
       <c r="Z10" s="5" t="inlineStr">
         <is>
@@ -2381,11 +2389,11 @@
         <v>22649882</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>23459424</v>
+        <v>23459422</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>ACC07</t>
+          <t>ACC05</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
@@ -2396,12 +2404,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -2416,7 +2424,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>ROSALINA FARIAS DIAS</t>
+          <t>DAMARIS RAQUELINA MALAQUIAS SARAIVA</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -2486,7 +2494,7 @@
         </is>
       </c>
       <c r="Y11" s="5" t="n">
-        <v>2243398445</v>
+        <v>2243398443</v>
       </c>
       <c r="Z11" s="5" t="inlineStr">
         <is>
@@ -2568,11 +2576,11 @@
         <v>22649882</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>23459425</v>
+        <v>23459423</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>ACC08</t>
+          <t>ACC06</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
@@ -2583,12 +2591,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -2603,7 +2611,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>LUANA CAROLINA LIMA DO NASCIMENTO</t>
+          <t>ANTONIA LETICIA DE SOUZA</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -2673,7 +2681,7 @@
         </is>
       </c>
       <c r="Y12" s="5" t="n">
-        <v>2243398446</v>
+        <v>2243398444</v>
       </c>
       <c r="Z12" s="5" t="inlineStr">
         <is>
@@ -2755,11 +2763,11 @@
         <v>22649882</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>23459426</v>
+        <v>23459424</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>ACC09</t>
+          <t>ACC07</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
@@ -2770,12 +2778,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -2790,7 +2798,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>RAQUEL PEREIRA DA SILVA</t>
+          <t>ROSALINA FARIAS DIAS</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -2860,7 +2868,7 @@
         </is>
       </c>
       <c r="Y13" s="5" t="n">
-        <v>2243398447</v>
+        <v>2243398445</v>
       </c>
       <c r="Z13" s="5" t="inlineStr">
         <is>
@@ -2942,11 +2950,11 @@
         <v>22649882</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>23459427</v>
+        <v>23459425</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ACC10</t>
+          <t>ACC08</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
@@ -2957,12 +2965,12 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -2977,7 +2985,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>DANIELA VAZ CAMILO</t>
+          <t>LUANA CAROLINA LIMA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -3047,7 +3055,7 @@
         </is>
       </c>
       <c r="Y14" s="5" t="n">
-        <v>2243398448</v>
+        <v>2243398446</v>
       </c>
       <c r="Z14" s="5" t="inlineStr">
         <is>
@@ -3129,11 +3137,11 @@
         <v>22649882</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>23459428</v>
+        <v>23459426</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>ACC11</t>
+          <t>ACC09</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
@@ -3144,12 +3152,12 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -3164,7 +3172,7 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>JESSICA RODRIGUES VIANA</t>
+          <t>RAQUEL PEREIRA DA SILVA</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -3234,7 +3242,7 @@
         </is>
       </c>
       <c r="Y15" s="5" t="n">
-        <v>2243398449</v>
+        <v>2243398447</v>
       </c>
       <c r="Z15" s="5" t="inlineStr">
         <is>
@@ -3316,11 +3324,11 @@
         <v>22649882</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>23459429</v>
+        <v>23459427</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ACC12</t>
+          <t>ACC10</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
@@ -3331,12 +3339,12 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -3351,7 +3359,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>JULIANA SILVA MACIEL</t>
+          <t>DANIELA VAZ CAMILO</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -3421,7 +3429,7 @@
         </is>
       </c>
       <c r="Y16" s="5" t="n">
-        <v>2243398450</v>
+        <v>2243398448</v>
       </c>
       <c r="Z16" s="5" t="inlineStr">
         <is>
@@ -3503,11 +3511,11 @@
         <v>22649882</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>23459430</v>
+        <v>23459428</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>ACC13</t>
+          <t>ACC11</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
@@ -3518,12 +3526,12 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -3538,7 +3546,7 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>RAISA SANTOS FERNANDES</t>
+          <t>JESSICA RODRIGUES VIANA</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -3608,7 +3616,7 @@
         </is>
       </c>
       <c r="Y17" s="5" t="n">
-        <v>2243398451</v>
+        <v>2243398449</v>
       </c>
       <c r="Z17" s="5" t="inlineStr">
         <is>
@@ -3690,11 +3698,11 @@
         <v>22649882</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>23459431</v>
+        <v>23459429</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>ACC14</t>
+          <t>ACC12</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
@@ -3705,12 +3713,12 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -3725,7 +3733,7 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>DANIELA APRIGIO TELES</t>
+          <t>JULIANA SILVA MACIEL</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -3795,7 +3803,7 @@
         </is>
       </c>
       <c r="Y18" s="5" t="n">
-        <v>2243398498</v>
+        <v>2243398450</v>
       </c>
       <c r="Z18" s="5" t="inlineStr">
         <is>
@@ -3877,11 +3885,11 @@
         <v>22649882</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>23459432</v>
+        <v>23459430</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>ACC15</t>
+          <t>ACC13</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
@@ -3892,12 +3900,12 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -3912,7 +3920,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>ANA CARLA BARROSO DE SOUSA TOMAZ</t>
+          <t>RAISA SANTOS FERNANDES</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
@@ -3982,7 +3990,7 @@
         </is>
       </c>
       <c r="Y19" s="5" t="n">
-        <v>2243398452</v>
+        <v>2243398451</v>
       </c>
       <c r="Z19" s="5" t="inlineStr">
         <is>
@@ -4064,11 +4072,11 @@
         <v>22649882</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>23459433</v>
+        <v>23459431</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>ACC16</t>
+          <t>ACC14</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
@@ -4079,12 +4087,12 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
@@ -4099,7 +4107,7 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>MARIA GISANE DOS SANTOS MACHADO</t>
+          <t>DANIELA APRIGIO TELES</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -4169,7 +4177,7 @@
         </is>
       </c>
       <c r="Y20" s="5" t="n">
-        <v>2243398453</v>
+        <v>2243398498</v>
       </c>
       <c r="Z20" s="5" t="inlineStr">
         <is>
@@ -4251,11 +4259,11 @@
         <v>22649882</v>
       </c>
       <c r="B21" s="5" t="n">
-        <v>23459434</v>
+        <v>23459432</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>ACC17</t>
+          <t>ACC15</t>
         </is>
       </c>
       <c r="D21" s="6" t="n">
@@ -4266,12 +4274,12 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -4286,7 +4294,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>RANGIELE DO CARMO ASSUNCAO</t>
+          <t>ANA CARLA BARROSO DE SOUSA TOMAZ</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
@@ -4356,7 +4364,7 @@
         </is>
       </c>
       <c r="Y21" s="5" t="n">
-        <v>2243398454</v>
+        <v>2243398452</v>
       </c>
       <c r="Z21" s="5" t="inlineStr">
         <is>
@@ -4438,11 +4446,11 @@
         <v>22649882</v>
       </c>
       <c r="B22" s="5" t="n">
-        <v>23459435</v>
+        <v>23459433</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>ACC18</t>
+          <t>ACC16</t>
         </is>
       </c>
       <c r="D22" s="6" t="n">
@@ -4453,12 +4461,12 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
@@ -4473,7 +4481,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>LUNARA SOUSA MOTA</t>
+          <t>MARIA GISANE DOS SANTOS MACHADO</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -4543,7 +4551,7 @@
         </is>
       </c>
       <c r="Y22" s="5" t="n">
-        <v>2243398455</v>
+        <v>2243398453</v>
       </c>
       <c r="Z22" s="5" t="inlineStr">
         <is>
@@ -4625,11 +4633,11 @@
         <v>22649882</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>23459436</v>
+        <v>23459434</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>ACC19</t>
+          <t>ACC17</t>
         </is>
       </c>
       <c r="D23" s="6" t="n">
@@ -4640,12 +4648,12 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -4660,7 +4668,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>HERLIA FERREIRA PEREIRA PALACIO</t>
+          <t>RANGIELE DO CARMO ASSUNCAO</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
@@ -4730,7 +4738,7 @@
         </is>
       </c>
       <c r="Y23" s="5" t="n">
-        <v>2243398456</v>
+        <v>2243398454</v>
       </c>
       <c r="Z23" s="5" t="inlineStr">
         <is>
@@ -4812,11 +4820,11 @@
         <v>22649882</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>23459437</v>
+        <v>23459435</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>ACC20</t>
+          <t>ACC18</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
@@ -4827,12 +4835,12 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -4847,7 +4855,7 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>GEANNE PIRES DE MESQUITA</t>
+          <t>LUNARA SOUSA MOTA</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -4917,7 +4925,7 @@
         </is>
       </c>
       <c r="Y24" s="5" t="n">
-        <v>2243398457</v>
+        <v>2243398455</v>
       </c>
       <c r="Z24" s="5" t="inlineStr">
         <is>
@@ -4999,11 +5007,11 @@
         <v>22649882</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>23459438</v>
+        <v>23459436</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>ACC21</t>
+          <t>ACC19</t>
         </is>
       </c>
       <c r="D25" s="6" t="n">
@@ -5014,12 +5022,12 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -5034,7 +5042,7 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>DANIELE FREITAS CAVALCANTE DE OLIVEIRA</t>
+          <t>HERLIA FERREIRA PEREIRA PALACIO</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
@@ -5104,7 +5112,7 @@
         </is>
       </c>
       <c r="Y25" s="5" t="n">
-        <v>2243398493</v>
+        <v>2243398456</v>
       </c>
       <c r="Z25" s="5" t="inlineStr">
         <is>
@@ -5186,11 +5194,11 @@
         <v>22649882</v>
       </c>
       <c r="B26" s="5" t="n">
-        <v>23459439</v>
+        <v>23459437</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>ACC22</t>
+          <t>ACC20</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
@@ -5201,12 +5209,12 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -5221,7 +5229,7 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>ADAILMA MENDES DOS SANTOS</t>
+          <t>GEANNE PIRES DE MESQUITA</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -5291,7 +5299,7 @@
         </is>
       </c>
       <c r="Y26" s="5" t="n">
-        <v>2243398459</v>
+        <v>2243398457</v>
       </c>
       <c r="Z26" s="5" t="inlineStr">
         <is>
@@ -5373,11 +5381,11 @@
         <v>22649882</v>
       </c>
       <c r="B27" s="5" t="n">
-        <v>23459440</v>
+        <v>23459438</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>ACC23</t>
+          <t>ACC21</t>
         </is>
       </c>
       <c r="D27" s="6" t="n">
@@ -5388,12 +5396,12 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -5408,7 +5416,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>KELEN CRISTINA MARTINS ALENCAR PINTO</t>
+          <t>DANIELE FREITAS CAVALCANTE DE OLIVEIRA</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
@@ -5478,7 +5486,7 @@
         </is>
       </c>
       <c r="Y27" s="5" t="n">
-        <v>2243398460</v>
+        <v>2243398493</v>
       </c>
       <c r="Z27" s="5" t="inlineStr">
         <is>
@@ -5560,11 +5568,11 @@
         <v>22649882</v>
       </c>
       <c r="B28" s="5" t="n">
-        <v>23459441</v>
+        <v>23459439</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>ACC24</t>
+          <t>ACC22</t>
         </is>
       </c>
       <c r="D28" s="6" t="n">
@@ -5575,12 +5583,12 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -5595,7 +5603,7 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>JORGEANA MORAIS MONTEIRO</t>
+          <t>ADAILMA MENDES DOS SANTOS</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -5665,7 +5673,7 @@
         </is>
       </c>
       <c r="Y28" s="5" t="n">
-        <v>2243398461</v>
+        <v>2243398459</v>
       </c>
       <c r="Z28" s="5" t="inlineStr">
         <is>
@@ -5747,11 +5755,11 @@
         <v>22649882</v>
       </c>
       <c r="B29" s="5" t="n">
-        <v>23459442</v>
+        <v>23459440</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>ACC25</t>
+          <t>ACC23</t>
         </is>
       </c>
       <c r="D29" s="6" t="n">
@@ -5762,12 +5770,12 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -5782,7 +5790,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>ANA CAROLINA CORREA</t>
+          <t>KELEN CRISTINA MARTINS ALENCAR PINTO</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -5852,7 +5860,7 @@
         </is>
       </c>
       <c r="Y29" s="5" t="n">
-        <v>2243398462</v>
+        <v>2243398460</v>
       </c>
       <c r="Z29" s="5" t="inlineStr">
         <is>
@@ -5934,11 +5942,11 @@
         <v>22649882</v>
       </c>
       <c r="B30" s="5" t="n">
-        <v>23459443</v>
+        <v>23459441</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>ACC26</t>
+          <t>ACC24</t>
         </is>
       </c>
       <c r="D30" s="6" t="n">
@@ -5949,12 +5957,12 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -5969,7 +5977,7 @@
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>IRLA GOMES DE SOUZA</t>
+          <t>JORGEANA MORAIS MONTEIRO</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -6039,7 +6047,7 @@
         </is>
       </c>
       <c r="Y30" s="5" t="n">
-        <v>2243398463</v>
+        <v>2243398461</v>
       </c>
       <c r="Z30" s="5" t="inlineStr">
         <is>
@@ -6121,11 +6129,11 @@
         <v>22649882</v>
       </c>
       <c r="B31" s="5" t="n">
-        <v>23459444</v>
+        <v>23459442</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>ACC27</t>
+          <t>ACC25</t>
         </is>
       </c>
       <c r="D31" s="6" t="n">
@@ -6136,12 +6144,12 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -6156,7 +6164,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>DAIANA MAGALHAES DE PAIVA</t>
+          <t>ANA CAROLINA CORREA</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
@@ -6226,7 +6234,7 @@
         </is>
       </c>
       <c r="Y31" s="5" t="n">
-        <v>2243398464</v>
+        <v>2243398462</v>
       </c>
       <c r="Z31" s="5" t="inlineStr">
         <is>
@@ -6308,11 +6316,11 @@
         <v>22649882</v>
       </c>
       <c r="B32" s="5" t="n">
-        <v>23459445</v>
+        <v>23459443</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>ACC28</t>
+          <t>ACC26</t>
         </is>
       </c>
       <c r="D32" s="6" t="n">
@@ -6323,12 +6331,12 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -6343,7 +6351,7 @@
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>FERNANDA HELENA ALVES DA ROCHA</t>
+          <t>IRLA GOMES DE SOUZA</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -6413,7 +6421,7 @@
         </is>
       </c>
       <c r="Y32" s="5" t="n">
-        <v>2243398465</v>
+        <v>2243398463</v>
       </c>
       <c r="Z32" s="5" t="inlineStr">
         <is>
@@ -6495,11 +6503,11 @@
         <v>22649882</v>
       </c>
       <c r="B33" s="5" t="n">
-        <v>23459446</v>
+        <v>23459444</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>ACC29</t>
+          <t>ACC27</t>
         </is>
       </c>
       <c r="D33" s="6" t="n">
@@ -6510,12 +6518,12 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
@@ -6530,7 +6538,7 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>KESSYA CARDOSO LIMA</t>
+          <t>DAIANA MAGALHAES DE PAIVA</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
@@ -6600,7 +6608,7 @@
         </is>
       </c>
       <c r="Y33" s="5" t="n">
-        <v>2243398466</v>
+        <v>2243398464</v>
       </c>
       <c r="Z33" s="5" t="inlineStr">
         <is>
@@ -6682,11 +6690,11 @@
         <v>22649882</v>
       </c>
       <c r="B34" s="5" t="n">
-        <v>23459447</v>
+        <v>23459445</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>ACC30</t>
+          <t>ACC28</t>
         </is>
       </c>
       <c r="D34" s="6" t="n">
@@ -6697,12 +6705,12 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
@@ -6717,7 +6725,7 @@
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>JESSICA CORREIA SALES</t>
+          <t>FERNANDA HELENA ALVES DA ROCHA</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
@@ -6787,7 +6795,7 @@
         </is>
       </c>
       <c r="Y34" s="5" t="n">
-        <v>2243398467</v>
+        <v>2243398465</v>
       </c>
       <c r="Z34" s="5" t="inlineStr">
         <is>
@@ -6869,11 +6877,11 @@
         <v>22649882</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>23459448</v>
+        <v>23459446</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>ACC31</t>
+          <t>ACC29</t>
         </is>
       </c>
       <c r="D35" s="6" t="n">
@@ -6884,12 +6892,12 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -6904,7 +6912,7 @@
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>MICHELLE PEREIRA DE OLIVEIRA</t>
+          <t>KESSYA CARDOSO LIMA</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
@@ -6974,7 +6982,7 @@
         </is>
       </c>
       <c r="Y35" s="5" t="n">
-        <v>2243398468</v>
+        <v>2243398466</v>
       </c>
       <c r="Z35" s="5" t="inlineStr">
         <is>
@@ -7056,11 +7064,11 @@
         <v>22649882</v>
       </c>
       <c r="B36" s="5" t="n">
-        <v>23459449</v>
+        <v>23459447</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>ACC32</t>
+          <t>ACC30</t>
         </is>
       </c>
       <c r="D36" s="6" t="n">
@@ -7071,12 +7079,12 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
@@ -7091,7 +7099,7 @@
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>NATALIA TAVARES DE ALMEIDA</t>
+          <t>JESSICA CORREIA SALES</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
@@ -7161,7 +7169,7 @@
         </is>
       </c>
       <c r="Y36" s="5" t="n">
-        <v>2243398469</v>
+        <v>2243398467</v>
       </c>
       <c r="Z36" s="5" t="inlineStr">
         <is>
@@ -7243,11 +7251,11 @@
         <v>22649882</v>
       </c>
       <c r="B37" s="5" t="n">
-        <v>23459450</v>
+        <v>23459448</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>ACC33</t>
+          <t>ACC31</t>
         </is>
       </c>
       <c r="D37" s="6" t="n">
@@ -7258,12 +7266,12 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
@@ -7278,7 +7286,7 @@
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>ANDREZZA RAYANNE ALVES DE ALMEIDA</t>
+          <t>MICHELLE PEREIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
@@ -7348,7 +7356,7 @@
         </is>
       </c>
       <c r="Y37" s="5" t="n">
-        <v>2243398470</v>
+        <v>2243398468</v>
       </c>
       <c r="Z37" s="5" t="inlineStr">
         <is>
@@ -7430,11 +7438,11 @@
         <v>22649882</v>
       </c>
       <c r="B38" s="5" t="n">
-        <v>23459451</v>
+        <v>23459449</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>ACC34</t>
+          <t>ACC32</t>
         </is>
       </c>
       <c r="D38" s="6" t="n">
@@ -7445,12 +7453,12 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
@@ -7465,7 +7473,7 @@
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>LILIAN KESSIA ALVES SIEBRA</t>
+          <t>NATALIA TAVARES DE ALMEIDA</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
@@ -7535,7 +7543,7 @@
         </is>
       </c>
       <c r="Y38" s="5" t="n">
-        <v>2243398471</v>
+        <v>2243398469</v>
       </c>
       <c r="Z38" s="5" t="inlineStr">
         <is>
@@ -7617,11 +7625,11 @@
         <v>22649882</v>
       </c>
       <c r="B39" s="5" t="n">
-        <v>23459452</v>
+        <v>23459450</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>ACC35</t>
+          <t>ACC33</t>
         </is>
       </c>
       <c r="D39" s="6" t="n">
@@ -7632,12 +7640,12 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
@@ -7652,7 +7660,7 @@
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>MONALISA DO NASCIMENTO RIBEIRO</t>
+          <t>ANDREZZA RAYANNE ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
@@ -7722,7 +7730,7 @@
         </is>
       </c>
       <c r="Y39" s="5" t="n">
-        <v>2243398472</v>
+        <v>2243398470</v>
       </c>
       <c r="Z39" s="5" t="inlineStr">
         <is>
@@ -7804,11 +7812,11 @@
         <v>22649882</v>
       </c>
       <c r="B40" s="5" t="n">
-        <v>23459453</v>
+        <v>23459451</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>ACC36</t>
+          <t>ACC34</t>
         </is>
       </c>
       <c r="D40" s="6" t="n">
@@ -7819,12 +7827,12 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
@@ -7839,7 +7847,7 @@
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>PRISCILA ADRIAN RODRIGUES</t>
+          <t>LILIAN KESSIA ALVES SIEBRA</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
@@ -7909,7 +7917,7 @@
         </is>
       </c>
       <c r="Y40" s="5" t="n">
-        <v>2243398473</v>
+        <v>2243398471</v>
       </c>
       <c r="Z40" s="5" t="inlineStr">
         <is>
@@ -7991,11 +7999,11 @@
         <v>22649882</v>
       </c>
       <c r="B41" s="5" t="n">
-        <v>23459454</v>
+        <v>23459452</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>ACC37</t>
+          <t>ACC35</t>
         </is>
       </c>
       <c r="D41" s="6" t="n">
@@ -8006,12 +8014,12 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
@@ -8026,7 +8034,7 @@
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>NATALIA FARIAS DE SOUSA</t>
+          <t>MONALISA DO NASCIMENTO RIBEIRO</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
@@ -8096,7 +8104,7 @@
         </is>
       </c>
       <c r="Y41" s="5" t="n">
-        <v>2243398474</v>
+        <v>2243398472</v>
       </c>
       <c r="Z41" s="5" t="inlineStr">
         <is>
@@ -8178,11 +8186,11 @@
         <v>22649882</v>
       </c>
       <c r="B42" s="5" t="n">
-        <v>23459455</v>
+        <v>23459453</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>ACC38</t>
+          <t>ACC36</t>
         </is>
       </c>
       <c r="D42" s="6" t="n">
@@ -8193,12 +8201,12 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
@@ -8213,7 +8221,7 @@
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>MARIANA MELO CAMURCA</t>
+          <t>PRISCILA ADRIAN RODRIGUES</t>
         </is>
       </c>
       <c r="K42" s="5" t="inlineStr">
@@ -8283,7 +8291,7 @@
         </is>
       </c>
       <c r="Y42" s="5" t="n">
-        <v>2243398475</v>
+        <v>2243398473</v>
       </c>
       <c r="Z42" s="5" t="inlineStr">
         <is>
@@ -8365,11 +8373,11 @@
         <v>22649882</v>
       </c>
       <c r="B43" s="5" t="n">
-        <v>23459456</v>
+        <v>23459454</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>ACC39</t>
+          <t>ACC37</t>
         </is>
       </c>
       <c r="D43" s="6" t="n">
@@ -8380,12 +8388,12 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
@@ -8400,7 +8408,7 @@
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>YOHANNA MARIA MENEZES DO NASCIMENTO</t>
+          <t>NATALIA FARIAS DE SOUSA</t>
         </is>
       </c>
       <c r="K43" s="5" t="inlineStr">
@@ -8470,7 +8478,7 @@
         </is>
       </c>
       <c r="Y43" s="5" t="n">
-        <v>2243398476</v>
+        <v>2243398474</v>
       </c>
       <c r="Z43" s="5" t="inlineStr">
         <is>
@@ -8552,11 +8560,11 @@
         <v>22649882</v>
       </c>
       <c r="B44" s="5" t="n">
-        <v>23459457</v>
+        <v>23459455</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>ACC40</t>
+          <t>ACC38</t>
         </is>
       </c>
       <c r="D44" s="6" t="n">
@@ -8567,12 +8575,12 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
@@ -8587,7 +8595,7 @@
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>MARIA ELINARA COSTA REBOUCAS</t>
+          <t>MARIANA MELO CAMURCA</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
@@ -8657,7 +8665,7 @@
         </is>
       </c>
       <c r="Y44" s="5" t="n">
-        <v>2243398477</v>
+        <v>2243398475</v>
       </c>
       <c r="Z44" s="5" t="inlineStr">
         <is>
@@ -8739,11 +8747,11 @@
         <v>22649882</v>
       </c>
       <c r="B45" s="5" t="n">
-        <v>23459458</v>
+        <v>23459456</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>ACC41</t>
+          <t>ACC39</t>
         </is>
       </c>
       <c r="D45" s="6" t="n">
@@ -8754,12 +8762,12 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
@@ -8774,7 +8782,7 @@
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>ANA MICHELLE LOUREIRO LOBO</t>
+          <t>YOHANNA MARIA MENEZES DO NASCIMENTO</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">
@@ -8844,7 +8852,7 @@
         </is>
       </c>
       <c r="Y45" s="5" t="n">
-        <v>2243398478</v>
+        <v>2243398476</v>
       </c>
       <c r="Z45" s="5" t="inlineStr">
         <is>
@@ -8926,11 +8934,11 @@
         <v>22649882</v>
       </c>
       <c r="B46" s="5" t="n">
-        <v>23459459</v>
+        <v>23459457</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>ACC42</t>
+          <t>ACC40</t>
         </is>
       </c>
       <c r="D46" s="6" t="n">
@@ -8941,12 +8949,12 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
@@ -8961,7 +8969,7 @@
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>MAIARA MARIA NASCIMENTO DE ARAUJO</t>
+          <t>MARIA ELINARA COSTA REBOUCAS</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
@@ -9031,7 +9039,7 @@
         </is>
       </c>
       <c r="Y46" s="5" t="n">
-        <v>2243398479</v>
+        <v>2243398477</v>
       </c>
       <c r="Z46" s="5" t="inlineStr">
         <is>
@@ -9113,11 +9121,11 @@
         <v>22649882</v>
       </c>
       <c r="B47" s="5" t="n">
-        <v>23459460</v>
+        <v>23459458</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>ACC43</t>
+          <t>ACC41</t>
         </is>
       </c>
       <c r="D47" s="6" t="n">
@@ -9128,12 +9136,12 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
@@ -9148,7 +9156,7 @@
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>THISIANIA ROMERO VIEIRA SOARES</t>
+          <t>ANA MICHELLE LOUREIRO LOBO</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
@@ -9218,7 +9226,7 @@
         </is>
       </c>
       <c r="Y47" s="5" t="n">
-        <v>2243398480</v>
+        <v>2243398478</v>
       </c>
       <c r="Z47" s="5" t="inlineStr">
         <is>
@@ -9300,11 +9308,11 @@
         <v>22649882</v>
       </c>
       <c r="B48" s="5" t="n">
-        <v>23459461</v>
+        <v>23459459</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>ACC44</t>
+          <t>ACC42</t>
         </is>
       </c>
       <c r="D48" s="6" t="n">
@@ -9315,12 +9323,12 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
@@ -9335,7 +9343,7 @@
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>CRISLANE ALENCARINA LIMA DA SILVA</t>
+          <t>MAIARA MARIA NASCIMENTO DE ARAUJO</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">
@@ -9405,7 +9413,7 @@
         </is>
       </c>
       <c r="Y48" s="5" t="n">
-        <v>2243398481</v>
+        <v>2243398479</v>
       </c>
       <c r="Z48" s="5" t="inlineStr">
         <is>
@@ -9487,11 +9495,11 @@
         <v>22649882</v>
       </c>
       <c r="B49" s="5" t="n">
-        <v>23459462</v>
+        <v>23459460</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>ACC45</t>
+          <t>ACC43</t>
         </is>
       </c>
       <c r="D49" s="6" t="n">
@@ -9502,12 +9510,12 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
@@ -9522,7 +9530,7 @@
       </c>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>PAULA AMANDA DO CARMO FERNANDES</t>
+          <t>THISIANIA ROMERO VIEIRA SOARES</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr">
@@ -9592,7 +9600,7 @@
         </is>
       </c>
       <c r="Y49" s="5" t="n">
-        <v>2243398482</v>
+        <v>2243398480</v>
       </c>
       <c r="Z49" s="5" t="inlineStr">
         <is>
@@ -9674,11 +9682,11 @@
         <v>22649882</v>
       </c>
       <c r="B50" s="5" t="n">
-        <v>23459463</v>
+        <v>23459461</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>ACC46</t>
+          <t>ACC44</t>
         </is>
       </c>
       <c r="D50" s="6" t="n">
@@ -9689,12 +9697,12 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
@@ -9709,7 +9717,7 @@
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>DIANA CARLA MORAES DOS SANTOS</t>
+          <t>CRISLANE ALENCARINA LIMA DA SILVA</t>
         </is>
       </c>
       <c r="K50" s="5" t="inlineStr">
@@ -9779,7 +9787,7 @@
         </is>
       </c>
       <c r="Y50" s="5" t="n">
-        <v>2243398483</v>
+        <v>2243398481</v>
       </c>
       <c r="Z50" s="5" t="inlineStr">
         <is>
@@ -9861,11 +9869,11 @@
         <v>22649882</v>
       </c>
       <c r="B51" s="5" t="n">
-        <v>23459465</v>
+        <v>23459462</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>ACC47</t>
+          <t>ACC45</t>
         </is>
       </c>
       <c r="D51" s="6" t="n">
@@ -9876,12 +9884,12 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
@@ -9896,7 +9904,7 @@
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>LUDMILA VIRNA OLIVEIRA FERNANDES</t>
+          <t>PAULA AMANDA DO CARMO FERNANDES</t>
         </is>
       </c>
       <c r="K51" s="5" t="inlineStr">
@@ -9966,7 +9974,7 @@
         </is>
       </c>
       <c r="Y51" s="5" t="n">
-        <v>2243398484</v>
+        <v>2243398482</v>
       </c>
       <c r="Z51" s="5" t="inlineStr">
         <is>
@@ -10048,11 +10056,11 @@
         <v>22649882</v>
       </c>
       <c r="B52" s="5" t="n">
-        <v>23459466</v>
+        <v>23459463</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>ACC48</t>
+          <t>ACC46</t>
         </is>
       </c>
       <c r="D52" s="6" t="n">
@@ -10063,12 +10071,12 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
@@ -10083,7 +10091,7 @@
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>CLAUDIANA HONORATO MIGUEL</t>
+          <t>DIANA CARLA MORAES DOS SANTOS</t>
         </is>
       </c>
       <c r="K52" s="5" t="inlineStr">
@@ -10153,7 +10161,7 @@
         </is>
       </c>
       <c r="Y52" s="5" t="n">
-        <v>2243398485</v>
+        <v>2243398483</v>
       </c>
       <c r="Z52" s="5" t="inlineStr">
         <is>
@@ -10235,11 +10243,11 @@
         <v>22649882</v>
       </c>
       <c r="B53" s="5" t="n">
-        <v>23459467</v>
+        <v>23459465</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>ACC49</t>
+          <t>ACC47</t>
         </is>
       </c>
       <c r="D53" s="6" t="n">
@@ -10250,12 +10258,12 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
@@ -10270,7 +10278,7 @@
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>SAN MILK RODRIGUES QUEIROZ</t>
+          <t>LUDMILA VIRNA OLIVEIRA FERNANDES</t>
         </is>
       </c>
       <c r="K53" s="5" t="inlineStr">
@@ -10340,7 +10348,7 @@
         </is>
       </c>
       <c r="Y53" s="5" t="n">
-        <v>2243398486</v>
+        <v>2243398484</v>
       </c>
       <c r="Z53" s="5" t="inlineStr">
         <is>
@@ -10422,11 +10430,11 @@
         <v>22649882</v>
       </c>
       <c r="B54" s="5" t="n">
-        <v>23459468</v>
+        <v>23459466</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>ACC50</t>
+          <t>ACC48</t>
         </is>
       </c>
       <c r="D54" s="6" t="n">
@@ -10437,12 +10445,12 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
@@ -10457,7 +10465,7 @@
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>JENNIFER MAINARA DA SILVA FACANHA</t>
+          <t>CLAUDIANA HONORATO MIGUEL</t>
         </is>
       </c>
       <c r="K54" s="5" t="inlineStr">
@@ -10527,7 +10535,7 @@
         </is>
       </c>
       <c r="Y54" s="5" t="n">
-        <v>2243398487</v>
+        <v>2243398485</v>
       </c>
       <c r="Z54" s="5" t="inlineStr">
         <is>
@@ -10609,11 +10617,11 @@
         <v>22649882</v>
       </c>
       <c r="B55" s="5" t="n">
-        <v>23459469</v>
+        <v>23459467</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>ACC51</t>
+          <t>ACC49</t>
         </is>
       </c>
       <c r="D55" s="6" t="n">
@@ -10624,12 +10632,12 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
@@ -10644,7 +10652,7 @@
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>THAIS MESQUITA GARCIA</t>
+          <t>SAN MILK RODRIGUES QUEIROZ</t>
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr">
@@ -10714,7 +10722,7 @@
         </is>
       </c>
       <c r="Y55" s="5" t="n">
-        <v>2243398488</v>
+        <v>2243398486</v>
       </c>
       <c r="Z55" s="5" t="inlineStr">
         <is>
@@ -10796,11 +10804,11 @@
         <v>22649882</v>
       </c>
       <c r="B56" s="5" t="n">
-        <v>23459470</v>
+        <v>23459468</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>ACC52</t>
+          <t>ACC50</t>
         </is>
       </c>
       <c r="D56" s="6" t="n">
@@ -10811,12 +10819,12 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
@@ -10831,7 +10839,7 @@
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>ARLETE CAVALCANTE ASSUNCAO</t>
+          <t>JENNIFER MAINARA DA SILVA FACANHA</t>
         </is>
       </c>
       <c r="K56" s="5" t="inlineStr">
@@ -10901,7 +10909,7 @@
         </is>
       </c>
       <c r="Y56" s="5" t="n">
-        <v>2243398489</v>
+        <v>2243398487</v>
       </c>
       <c r="Z56" s="5" t="inlineStr">
         <is>
@@ -10983,11 +10991,11 @@
         <v>22649882</v>
       </c>
       <c r="B57" s="5" t="n">
-        <v>23459471</v>
+        <v>23459469</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>ACC53</t>
+          <t>ACC51</t>
         </is>
       </c>
       <c r="D57" s="6" t="n">
@@ -10998,12 +11006,12 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
@@ -11018,7 +11026,7 @@
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>KELIANE DA SILVA SOARES</t>
+          <t>THAIS MESQUITA GARCIA</t>
         </is>
       </c>
       <c r="K57" s="5" t="inlineStr">
@@ -11088,7 +11096,7 @@
         </is>
       </c>
       <c r="Y57" s="5" t="n">
-        <v>2243398490</v>
+        <v>2243398488</v>
       </c>
       <c r="Z57" s="5" t="inlineStr">
         <is>
@@ -11170,11 +11178,11 @@
         <v>22649882</v>
       </c>
       <c r="B58" s="5" t="n">
-        <v>23459472</v>
+        <v>23459470</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>ACC54</t>
+          <t>ACC52</t>
         </is>
       </c>
       <c r="D58" s="6" t="n">
@@ -11185,12 +11193,12 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr">
@@ -11205,7 +11213,7 @@
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>MIKAELLA DOS SANTOS ALVES</t>
+          <t>ARLETE CAVALCANTE ASSUNCAO</t>
         </is>
       </c>
       <c r="K58" s="5" t="inlineStr">
@@ -11275,7 +11283,7 @@
         </is>
       </c>
       <c r="Y58" s="5" t="n">
-        <v>2243398491</v>
+        <v>2243398489</v>
       </c>
       <c r="Z58" s="5" t="inlineStr">
         <is>
@@ -11357,11 +11365,11 @@
         <v>22649882</v>
       </c>
       <c r="B59" s="5" t="n">
-        <v>23459473</v>
+        <v>23459471</v>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>ACC55</t>
+          <t>ACC53</t>
         </is>
       </c>
       <c r="D59" s="6" t="n">
@@ -11372,12 +11380,12 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr">
@@ -11392,7 +11400,7 @@
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>ANNA CLARA DOMINGOS ALVES</t>
+          <t>KELIANE DA SILVA SOARES</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
@@ -11462,7 +11470,7 @@
         </is>
       </c>
       <c r="Y59" s="5" t="n">
-        <v>2243398492</v>
+        <v>2243398490</v>
       </c>
       <c r="Z59" s="5" t="inlineStr">
         <is>
@@ -11544,11 +11552,11 @@
         <v>22649882</v>
       </c>
       <c r="B60" s="5" t="n">
-        <v>23459474</v>
+        <v>23459472</v>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>ACC56</t>
+          <t>ACC54</t>
         </is>
       </c>
       <c r="D60" s="6" t="n">
@@ -11559,12 +11567,12 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
@@ -11579,7 +11587,7 @@
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>FRANCISCA ERICA COSTA DE MENEZES</t>
+          <t>MIKAELLA DOS SANTOS ALVES</t>
         </is>
       </c>
       <c r="K60" s="5" t="inlineStr">
@@ -11649,7 +11657,7 @@
         </is>
       </c>
       <c r="Y60" s="5" t="n">
-        <v>2243398493</v>
+        <v>2243398491</v>
       </c>
       <c r="Z60" s="5" t="inlineStr">
         <is>
@@ -11731,11 +11739,11 @@
         <v>22649882</v>
       </c>
       <c r="B61" s="5" t="n">
-        <v>23459475</v>
+        <v>23459473</v>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>ACC57</t>
+          <t>ACC55</t>
         </is>
       </c>
       <c r="D61" s="6" t="n">
@@ -11746,12 +11754,12 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
@@ -11766,7 +11774,7 @@
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>LUIZIANNE MARIA GONCALVES DE ALENCAR</t>
+          <t>ANNA CLARA DOMINGOS ALVES</t>
         </is>
       </c>
       <c r="K61" s="5" t="inlineStr">
@@ -11836,7 +11844,7 @@
         </is>
       </c>
       <c r="Y61" s="5" t="n">
-        <v>2243398494</v>
+        <v>2243398492</v>
       </c>
       <c r="Z61" s="5" t="inlineStr">
         <is>
@@ -11918,11 +11926,11 @@
         <v>22649882</v>
       </c>
       <c r="B62" s="5" t="n">
-        <v>23459476</v>
+        <v>23459474</v>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>ACC58</t>
+          <t>ACC56</t>
         </is>
       </c>
       <c r="D62" s="6" t="n">
@@ -11933,12 +11941,12 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
@@ -11953,7 +11961,7 @@
       </c>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>LUAN MIKAEL DE SOUSA PEREIRA</t>
+          <t>FRANCISCA ERICA COSTA DE MENEZES</t>
         </is>
       </c>
       <c r="K62" s="5" t="inlineStr">
@@ -12023,7 +12031,7 @@
         </is>
       </c>
       <c r="Y62" s="5" t="n">
-        <v>2243398495</v>
+        <v>2243398493</v>
       </c>
       <c r="Z62" s="5" t="inlineStr">
         <is>
@@ -12105,11 +12113,11 @@
         <v>22649882</v>
       </c>
       <c r="B63" s="5" t="n">
-        <v>23459477</v>
+        <v>23459475</v>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>ACC59</t>
+          <t>ACC57</t>
         </is>
       </c>
       <c r="D63" s="6" t="n">
@@ -12120,12 +12128,12 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr">
@@ -12140,7 +12148,7 @@
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>ANA CAROLINA MOREIRA QUEIROZ</t>
+          <t>LUIZIANNE MARIA GONCALVES DE ALENCAR</t>
         </is>
       </c>
       <c r="K63" s="5" t="inlineStr">
@@ -12210,7 +12218,7 @@
         </is>
       </c>
       <c r="Y63" s="5" t="n">
-        <v>2243398496</v>
+        <v>2243398494</v>
       </c>
       <c r="Z63" s="5" t="inlineStr">
         <is>
@@ -12292,11 +12300,11 @@
         <v>22649882</v>
       </c>
       <c r="B64" s="5" t="n">
-        <v>23459478</v>
+        <v>23459476</v>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>ACC60</t>
+          <t>ACC58</t>
         </is>
       </c>
       <c r="D64" s="6" t="n">
@@ -12307,12 +12315,12 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr">
@@ -12327,7 +12335,7 @@
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>GABRIEL DA SILVA ROCHA</t>
+          <t>LUAN MIKAEL DE SOUSA PEREIRA</t>
         </is>
       </c>
       <c r="K64" s="5" t="inlineStr">
@@ -12397,7 +12405,7 @@
         </is>
       </c>
       <c r="Y64" s="5" t="n">
-        <v>2243398497</v>
+        <v>2243398495</v>
       </c>
       <c r="Z64" s="5" t="inlineStr">
         <is>
@@ -12469,6 +12477,380 @@
         </is>
       </c>
       <c r="AQ64" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n">
+        <v>22649882</v>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>23459477</v>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>ACC59</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>45868.40885416666</v>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>45868.41748842593</v>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>HNMBIK</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>ANA CAROLINA MOREIRA QUEIROZ</t>
+        </is>
+      </c>
+      <c r="K65" s="5" t="inlineStr">
+        <is>
+          <t>Jaqueline Rodrigues Teixeira</t>
+        </is>
+      </c>
+      <c r="L65" s="5" t="inlineStr">
+        <is>
+          <t>Jaqueline Rodrigues Teixeira</t>
+        </is>
+      </c>
+      <c r="M65" s="6" t="n">
+        <v>45867</v>
+      </c>
+      <c r="N65" s="5" t="n">
+        <v>4801518571</v>
+      </c>
+      <c r="O65" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P65" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q65" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R65" s="5" t="inlineStr">
+        <is>
+          <t>Faturado</t>
+        </is>
+      </c>
+      <c r="S65" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T65" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U65" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Diageo</t>
+        </is>
+      </c>
+      <c r="V65" s="5" t="inlineStr">
+        <is>
+          <t>Diageo Brasil</t>
+        </is>
+      </c>
+      <c r="W65" s="5" t="inlineStr">
+        <is>
+          <t>Cliente FEE no POS</t>
+        </is>
+      </c>
+      <c r="X65" s="5" t="inlineStr">
+        <is>
+          <t>Latam Airlines Brasil</t>
+        </is>
+      </c>
+      <c r="Y65" s="5" t="n">
+        <v>2243398496</v>
+      </c>
+      <c r="Z65" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+      <c r="AA65" s="5" t="n">
+        <v>167526</v>
+      </c>
+      <c r="AB65" s="5" t="n">
+        <v>683.05</v>
+      </c>
+      <c r="AC65" s="5" t="n">
+        <v>31.44</v>
+      </c>
+      <c r="AD65" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE65" s="5" t="n">
+        <v>68.25</v>
+      </c>
+      <c r="AF65" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG65" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH65" s="5" t="n">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="AI65" s="5" t="inlineStr">
+        <is>
+          <t>Reserva importada via planilha. Solicitação: |PC:</t>
+        </is>
+      </c>
+      <c r="AJ65" s="5" t="inlineStr">
+        <is>
+          <t>Verificação de bilhetes: Bilhete 2243398493 já sendo utilizado para este fornecedor.</t>
+        </is>
+      </c>
+      <c r="AK65" s="5" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="AL65" s="5" t="inlineStr">
+        <is>
+          <t>Bilhete duplicado</t>
+        </is>
+      </c>
+      <c r="AM65" s="5" t="inlineStr">
+        <is>
+          <t>Bilhete Já Contabilizado</t>
+        </is>
+      </c>
+      <c r="AN65" s="5" t="inlineStr">
+        <is>
+          <t>Duplicidade de Contabilização</t>
+        </is>
+      </c>
+      <c r="AO65" s="5" t="inlineStr">
+        <is>
+          <t>Qualidade dos dados</t>
+        </is>
+      </c>
+      <c r="AP65" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+      <c r="AQ65" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="n">
+        <v>22649882</v>
+      </c>
+      <c r="B66" s="5" t="n">
+        <v>23459478</v>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>ACC60</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="n">
+        <v>45868.40885416666</v>
+      </c>
+      <c r="E66" s="6" t="n">
+        <v>45868.41748842593</v>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>HNMBIK</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>GABRIEL DA SILVA ROCHA</t>
+        </is>
+      </c>
+      <c r="K66" s="5" t="inlineStr">
+        <is>
+          <t>Jaqueline Rodrigues Teixeira</t>
+        </is>
+      </c>
+      <c r="L66" s="5" t="inlineStr">
+        <is>
+          <t>Jaqueline Rodrigues Teixeira</t>
+        </is>
+      </c>
+      <c r="M66" s="6" t="n">
+        <v>45867</v>
+      </c>
+      <c r="N66" s="5" t="n">
+        <v>4801518571</v>
+      </c>
+      <c r="O66" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P66" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q66" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R66" s="5" t="inlineStr">
+        <is>
+          <t>Faturado</t>
+        </is>
+      </c>
+      <c r="S66" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T66" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U66" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Diageo</t>
+        </is>
+      </c>
+      <c r="V66" s="5" t="inlineStr">
+        <is>
+          <t>Diageo Brasil</t>
+        </is>
+      </c>
+      <c r="W66" s="5" t="inlineStr">
+        <is>
+          <t>Cliente FEE no POS</t>
+        </is>
+      </c>
+      <c r="X66" s="5" t="inlineStr">
+        <is>
+          <t>Latam Airlines Brasil</t>
+        </is>
+      </c>
+      <c r="Y66" s="5" t="n">
+        <v>2243398497</v>
+      </c>
+      <c r="Z66" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+      <c r="AA66" s="5" t="n">
+        <v>167526</v>
+      </c>
+      <c r="AB66" s="5" t="n">
+        <v>683.05</v>
+      </c>
+      <c r="AC66" s="5" t="n">
+        <v>31.44</v>
+      </c>
+      <c r="AD66" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE66" s="5" t="n">
+        <v>68.25</v>
+      </c>
+      <c r="AF66" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG66" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH66" s="5" t="n">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="AI66" s="5" t="inlineStr">
+        <is>
+          <t>Reserva importada via planilha. Solicitação: |PC:</t>
+        </is>
+      </c>
+      <c r="AJ66" s="5" t="inlineStr">
+        <is>
+          <t>Verificação de bilhetes: Bilhete 2243398493 já sendo utilizado para este fornecedor.</t>
+        </is>
+      </c>
+      <c r="AK66" s="5" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="AL66" s="5" t="inlineStr">
+        <is>
+          <t>Bilhete duplicado</t>
+        </is>
+      </c>
+      <c r="AM66" s="5" t="inlineStr">
+        <is>
+          <t>Bilhete Já Contabilizado</t>
+        </is>
+      </c>
+      <c r="AN66" s="5" t="inlineStr">
+        <is>
+          <t>Duplicidade de Contabilização</t>
+        </is>
+      </c>
+      <c r="AO66" s="5" t="inlineStr">
+        <is>
+          <t>Qualidade dos dados</t>
+        </is>
+      </c>
+      <c r="AP66" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+      <c r="AQ66" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>

</xml_diff>

<commit_message>
Update report paths and add new PDF reports
Refactored file paths in 4-envio_relatorios.py to use the data_path variable for consistency. Updated several Excel report files and added new PDF reports for 06.08.2025, 07.08.2025, and 08.08.2025.
</commit_message>
<xml_diff>
--- a/Integration-Quality/EMPRESAS/Relatorio - INOVENTS.xlsx
+++ b/Integration-Quality/EMPRESAS/Relatorio - INOVENTS.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ66"/>
+  <dimension ref="A1:AQ65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,10 +695,10 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>22679559</v>
+        <v>22691840</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>23484064</v>
+        <v>23494864</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
@@ -706,10 +706,10 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>45873.65900462963</v>
+        <v>45875.3809375</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>45873.67644675926</v>
+        <v>45875.38268518518</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>B3NZNT</t>
+          <t>5GDF7M</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -733,21 +733,21 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>BUENO BARBOSA/RENATA</t>
+          <t>SERVICO</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Danny Junqueira Martins</t>
+          <t>Elaine Cristina Martins</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Danny Junqueira Martins</t>
+          <t>Elaine Cristina Martins</t>
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>45873.65833333333</v>
+        <v>45875.38055555556</v>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
@@ -776,7 +776,7 @@
       </c>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>Aéreo</t>
+          <t>Serviço</t>
         </is>
       </c>
       <c r="T2" s="5" t="inlineStr">
@@ -786,12 +786,12 @@
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>Grupo Jti</t>
+          <t>-</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>Jti Distribuidora - Sao Paulo - Vila Nova Conceicao</t>
+          <t>Claro S/a</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -801,27 +801,27 @@
       </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="Y2" s="5" t="n">
-        <v>2971556787</v>
+          <t>Ciclo Academy</t>
+        </is>
+      </c>
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>
       </c>
-      <c r="AA2" s="5" t="inlineStr">
-        <is>
-          <t>ID152723</t>
-        </is>
+      <c r="AA2" s="5" t="n">
+        <v>170240</v>
       </c>
       <c r="AB2" s="5" t="n">
-        <v>6420.23</v>
+        <v>16875</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>464.43</v>
+        <v>0</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
@@ -836,7 +836,7 @@
         <v>0</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>655.21</v>
+        <v>0</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
@@ -845,7 +845,7 @@
       </c>
       <c r="AJ2" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2971556787 já sendo utilizado para este fornecedor.</t>
+          <t>Necessário cadastrar um contrato para o cliente ""</t>
         </is>
       </c>
       <c r="AK2" s="5" t="inlineStr">
@@ -855,17 +855,17 @@
       </c>
       <c r="AL2" s="5" t="inlineStr">
         <is>
-          <t>Bilhete duplicado</t>
+          <t>Contrato de fornecedor</t>
         </is>
       </c>
       <c r="AM2" s="5" t="inlineStr">
         <is>
-          <t>Bilhete Já Contabilizado</t>
+          <t>Análise Cadastro</t>
         </is>
       </c>
       <c r="AN2" s="5" t="inlineStr">
         <is>
-          <t>Duplicidade de Contabilização</t>
+          <t>Dados do Fornecedor</t>
         </is>
       </c>
       <c r="AO2" s="5" t="inlineStr">
@@ -886,10 +886,10 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>22679559</v>
+        <v>22691840</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>23484078</v>
+        <v>23494866</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -897,10 +897,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>45873.65900462963</v>
+        <v>45875.3809375</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>45873.67644675926</v>
+        <v>45875.38268518518</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>B3NZNT</t>
+          <t>5GDF7M</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -924,21 +924,21 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>SIMOES BARBOSA/FRANCISCO</t>
+          <t>FEE+TAXAS</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Danny Junqueira Martins</t>
+          <t>Elaine Cristina Martins</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Danny Junqueira Martins</t>
+          <t>Elaine Cristina Martins</t>
         </is>
       </c>
       <c r="M3" s="6" t="n">
-        <v>45873.65833333333</v>
+        <v>45875.38055555556</v>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
@@ -967,7 +967,7 @@
       </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
-          <t>Aéreo</t>
+          <t>Serviço</t>
         </is>
       </c>
       <c r="T3" s="5" t="inlineStr">
@@ -977,12 +977,12 @@
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>Grupo Jti</t>
+          <t>-</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>Jti Distribuidora - Sao Paulo - Vila Nova Conceicao</t>
+          <t>Claro S/a</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
@@ -992,27 +992,27 @@
       </c>
       <c r="X3" s="5" t="inlineStr">
         <is>
-          <t>Iberia</t>
-        </is>
-      </c>
-      <c r="Y3" s="5" t="n">
-        <v>2971556785</v>
+          <t>Ciclo Academy</t>
+        </is>
+      </c>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>
       </c>
-      <c r="AA3" s="5" t="inlineStr">
-        <is>
-          <t>ID152723</t>
-        </is>
+      <c r="AA3" s="5" t="n">
+        <v>170240</v>
       </c>
       <c r="AB3" s="5" t="n">
-        <v>6420.23</v>
+        <v>0</v>
       </c>
       <c r="AC3" s="5" t="n">
-        <v>464.43</v>
+        <v>0</v>
       </c>
       <c r="AD3" s="5" t="n">
         <v>0</v>
@@ -1027,7 +1027,7 @@
         <v>0</v>
       </c>
       <c r="AH3" s="5" t="n">
-        <v>655.21</v>
+        <v>2568.04</v>
       </c>
       <c r="AI3" s="5" t="inlineStr">
         <is>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="AJ3" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2971556787 já sendo utilizado para este fornecedor.</t>
+          <t>Necessário cadastrar um contrato para o cliente ""</t>
         </is>
       </c>
       <c r="AK3" s="5" t="inlineStr">
@@ -1046,17 +1046,17 @@
       </c>
       <c r="AL3" s="5" t="inlineStr">
         <is>
-          <t>Bilhete duplicado</t>
+          <t>Contrato de fornecedor</t>
         </is>
       </c>
       <c r="AM3" s="5" t="inlineStr">
         <is>
-          <t>Bilhete Já Contabilizado</t>
+          <t>Análise Cadastro</t>
         </is>
       </c>
       <c r="AN3" s="5" t="inlineStr">
         <is>
-          <t>Duplicidade de Contabilização</t>
+          <t>Dados do Fornecedor</t>
         </is>
       </c>
       <c r="AO3" s="5" t="inlineStr">
@@ -1077,10 +1077,10 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>22649878</v>
+        <v>22649882</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>23459408</v>
+        <v>23459418</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -1088,24 +1088,24 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>45868.40864583333</v>
+        <v>45868.40885416666</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>45868.41383101852</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>EGHULO</t>
+          <t>HNMBIK</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>AMANDA MAYARA HENRIQUE DE OLIVEIRA</t>
+          <t>BARBARA MAGALHAES</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1185,7 +1185,7 @@
         </is>
       </c>
       <c r="Y4" s="5" t="n">
-        <v>2243394807</v>
+        <v>2243398439</v>
       </c>
       <c r="Z4" s="5" t="inlineStr">
         <is>
@@ -1196,16 +1196,16 @@
         <v>167526</v>
       </c>
       <c r="AB4" s="5" t="n">
-        <v>1542.36</v>
+        <v>683.05</v>
       </c>
       <c r="AC4" s="5" t="n">
-        <v>77.64</v>
+        <v>31.44</v>
       </c>
       <c r="AD4" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE4" s="5" t="n">
-        <v>154.23</v>
+        <v>68.25</v>
       </c>
       <c r="AF4" s="5" t="n">
         <v>0</v>
@@ -1214,7 +1214,7 @@
         <v>0</v>
       </c>
       <c r="AH4" s="5" t="n">
-        <v>192.85</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="AI4" s="5" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="AJ4" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2243394807 já sendo utilizado para este fornecedor.</t>
+          <t>Verificação de bilhetes: Bilhete 2243398493 já sendo utilizado para este fornecedor.</t>
         </is>
       </c>
       <c r="AK4" s="5" t="inlineStr">
@@ -1264,10 +1264,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>22649878</v>
+        <v>22649882</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>23459409</v>
+        <v>23459419</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -1275,24 +1275,24 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>45868.40864583333</v>
+        <v>45868.40885416666</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>45868.41383101852</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>EGHULO</t>
+          <t>HNMBIK</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>MARIA LUIZA PEREIRA LIRA</t>
+          <t>JAMYLE PINHEIRO FACANHA CAVALCANTE</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -1372,7 +1372,7 @@
         </is>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>2243394807</v>
+        <v>2243398440</v>
       </c>
       <c r="Z5" s="5" t="inlineStr">
         <is>
@@ -1383,16 +1383,16 @@
         <v>167526</v>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>1542.36</v>
+        <v>683.05</v>
       </c>
       <c r="AC5" s="5" t="n">
-        <v>77.64</v>
+        <v>31.44</v>
       </c>
       <c r="AD5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE5" s="5" t="n">
-        <v>154.23</v>
+        <v>68.25</v>
       </c>
       <c r="AF5" s="5" t="n">
         <v>0</v>
@@ -1401,7 +1401,7 @@
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="n">
-        <v>192.85</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="AI5" s="5" t="inlineStr">
         <is>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="AJ5" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2243394807 já sendo utilizado para este fornecedor.</t>
+          <t>Verificação de bilhetes: Bilhete 2243398493 já sendo utilizado para este fornecedor.</t>
         </is>
       </c>
       <c r="AK5" s="5" t="inlineStr">
@@ -1451,10 +1451,10 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>22649878</v>
+        <v>22649882</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>23459410</v>
+        <v>23459420</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -1462,24 +1462,24 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>45868.40864583333</v>
+        <v>45868.40885416666</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>45868.41383101852</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>EGHULO</t>
+          <t>HNMBIK</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>EVERTON NUNES DA SILVA</t>
+          <t>CHRISTIANE GURGEL DO AMARAL CHAVES</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="Y6" s="5" t="n">
-        <v>2243394807</v>
+        <v>2243398441</v>
       </c>
       <c r="Z6" s="5" t="inlineStr">
         <is>
@@ -1570,16 +1570,16 @@
         <v>167526</v>
       </c>
       <c r="AB6" s="5" t="n">
-        <v>1542.36</v>
+        <v>683.05</v>
       </c>
       <c r="AC6" s="5" t="n">
-        <v>77.64</v>
+        <v>31.44</v>
       </c>
       <c r="AD6" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE6" s="5" t="n">
-        <v>154.23</v>
+        <v>68.25</v>
       </c>
       <c r="AF6" s="5" t="n">
         <v>0</v>
@@ -1588,7 +1588,7 @@
         <v>0</v>
       </c>
       <c r="AH6" s="5" t="n">
-        <v>192.85</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="AI6" s="5" t="inlineStr">
         <is>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="AJ6" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2243394807 já sendo utilizado para este fornecedor.</t>
+          <t>Verificação de bilhetes: Bilhete 2243398493 já sendo utilizado para este fornecedor.</t>
         </is>
       </c>
       <c r="AK6" s="5" t="inlineStr">
@@ -1641,27 +1641,27 @@
         <v>22649882</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>23459418</v>
+        <v>23459421</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>ACC01</t>
+          <t>ACC04</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>BARBARA MAGALHAES</t>
+          <t>HELEN LIDIA MENDES</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="Y7" s="5" t="n">
-        <v>2243398439</v>
+        <v>2243398442</v>
       </c>
       <c r="Z7" s="5" t="inlineStr">
         <is>
@@ -1828,27 +1828,27 @@
         <v>22649882</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>23459419</v>
+        <v>23459422</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC05</t>
         </is>
       </c>
       <c r="D8" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>JAMYLE PINHEIRO FACANHA CAVALCANTE</t>
+          <t>DAMARIS RAQUELINA MALAQUIAS SARAIVA</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="Y8" s="5" t="n">
-        <v>2243398440</v>
+        <v>2243398443</v>
       </c>
       <c r="Z8" s="5" t="inlineStr">
         <is>
@@ -2015,27 +2015,27 @@
         <v>22649882</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>23459420</v>
+        <v>23459423</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>ACC03</t>
+          <t>ACC06</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>CHRISTIANE GURGEL DO AMARAL CHAVES</t>
+          <t>ANTONIA LETICIA DE SOUZA</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -2120,7 +2120,7 @@
         </is>
       </c>
       <c r="Y9" s="5" t="n">
-        <v>2243398441</v>
+        <v>2243398444</v>
       </c>
       <c r="Z9" s="5" t="inlineStr">
         <is>
@@ -2202,27 +2202,27 @@
         <v>22649882</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>23459421</v>
+        <v>23459424</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ACC04</t>
+          <t>ACC07</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>HELEN LIDIA MENDES</t>
+          <t>ROSALINA FARIAS DIAS</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -2307,7 +2307,7 @@
         </is>
       </c>
       <c r="Y10" s="5" t="n">
-        <v>2243398442</v>
+        <v>2243398445</v>
       </c>
       <c r="Z10" s="5" t="inlineStr">
         <is>
@@ -2389,27 +2389,27 @@
         <v>22649882</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>23459422</v>
+        <v>23459425</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>ACC05</t>
+          <t>ACC08</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>DAMARIS RAQUELINA MALAQUIAS SARAIVA</t>
+          <t>LUANA CAROLINA LIMA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -2494,7 +2494,7 @@
         </is>
       </c>
       <c r="Y11" s="5" t="n">
-        <v>2243398443</v>
+        <v>2243398446</v>
       </c>
       <c r="Z11" s="5" t="inlineStr">
         <is>
@@ -2576,27 +2576,27 @@
         <v>22649882</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>23459423</v>
+        <v>23459426</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>ACC06</t>
+          <t>ACC09</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>ANTONIA LETICIA DE SOUZA</t>
+          <t>RAQUEL PEREIRA DA SILVA</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="Y12" s="5" t="n">
-        <v>2243398444</v>
+        <v>2243398447</v>
       </c>
       <c r="Z12" s="5" t="inlineStr">
         <is>
@@ -2763,27 +2763,27 @@
         <v>22649882</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>23459424</v>
+        <v>23459427</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>ACC07</t>
+          <t>ACC10</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>ROSALINA FARIAS DIAS</t>
+          <t>DANIELA VAZ CAMILO</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -2868,7 +2868,7 @@
         </is>
       </c>
       <c r="Y13" s="5" t="n">
-        <v>2243398445</v>
+        <v>2243398448</v>
       </c>
       <c r="Z13" s="5" t="inlineStr">
         <is>
@@ -2950,27 +2950,27 @@
         <v>22649882</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>23459425</v>
+        <v>23459428</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ACC08</t>
+          <t>ACC11</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>LUANA CAROLINA LIMA DO NASCIMENTO</t>
+          <t>JESSICA RODRIGUES VIANA</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="Y14" s="5" t="n">
-        <v>2243398446</v>
+        <v>2243398449</v>
       </c>
       <c r="Z14" s="5" t="inlineStr">
         <is>
@@ -3137,27 +3137,27 @@
         <v>22649882</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>23459426</v>
+        <v>23459429</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>ACC09</t>
+          <t>ACC12</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>RAQUEL PEREIRA DA SILVA</t>
+          <t>JULIANA SILVA MACIEL</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -3242,7 +3242,7 @@
         </is>
       </c>
       <c r="Y15" s="5" t="n">
-        <v>2243398447</v>
+        <v>2243398450</v>
       </c>
       <c r="Z15" s="5" t="inlineStr">
         <is>
@@ -3324,27 +3324,27 @@
         <v>22649882</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>23459427</v>
+        <v>23459430</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ACC10</t>
+          <t>ACC13</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>DANIELA VAZ CAMILO</t>
+          <t>RAISA SANTOS FERNANDES</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -3429,7 +3429,7 @@
         </is>
       </c>
       <c r="Y16" s="5" t="n">
-        <v>2243398448</v>
+        <v>2243398451</v>
       </c>
       <c r="Z16" s="5" t="inlineStr">
         <is>
@@ -3511,27 +3511,27 @@
         <v>22649882</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>23459428</v>
+        <v>23459431</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>ACC11</t>
+          <t>ACC14</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>JESSICA RODRIGUES VIANA</t>
+          <t>DANIELA APRIGIO TELES</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -3616,7 +3616,7 @@
         </is>
       </c>
       <c r="Y17" s="5" t="n">
-        <v>2243398449</v>
+        <v>2243398498</v>
       </c>
       <c r="Z17" s="5" t="inlineStr">
         <is>
@@ -3698,27 +3698,27 @@
         <v>22649882</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>23459429</v>
+        <v>23459432</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>ACC12</t>
+          <t>ACC15</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -3733,7 +3733,7 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>JULIANA SILVA MACIEL</t>
+          <t>ANA CARLA BARROSO DE SOUSA TOMAZ</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -3803,7 +3803,7 @@
         </is>
       </c>
       <c r="Y18" s="5" t="n">
-        <v>2243398450</v>
+        <v>2243398452</v>
       </c>
       <c r="Z18" s="5" t="inlineStr">
         <is>
@@ -3885,27 +3885,27 @@
         <v>22649882</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>23459430</v>
+        <v>23459433</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>ACC13</t>
+          <t>ACC16</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>RAISA SANTOS FERNANDES</t>
+          <t>MARIA GISANE DOS SANTOS MACHADO</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
@@ -3990,7 +3990,7 @@
         </is>
       </c>
       <c r="Y19" s="5" t="n">
-        <v>2243398451</v>
+        <v>2243398453</v>
       </c>
       <c r="Z19" s="5" t="inlineStr">
         <is>
@@ -4072,27 +4072,27 @@
         <v>22649882</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>23459431</v>
+        <v>23459434</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>ACC14</t>
+          <t>ACC17</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>DANIELA APRIGIO TELES</t>
+          <t>RANGIELE DO CARMO ASSUNCAO</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -4177,7 +4177,7 @@
         </is>
       </c>
       <c r="Y20" s="5" t="n">
-        <v>2243398498</v>
+        <v>2243398454</v>
       </c>
       <c r="Z20" s="5" t="inlineStr">
         <is>
@@ -4259,27 +4259,27 @@
         <v>22649882</v>
       </c>
       <c r="B21" s="5" t="n">
-        <v>23459432</v>
+        <v>23459435</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>ACC15</t>
+          <t>ACC18</t>
         </is>
       </c>
       <c r="D21" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>ANA CARLA BARROSO DE SOUSA TOMAZ</t>
+          <t>LUNARA SOUSA MOTA</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
@@ -4364,7 +4364,7 @@
         </is>
       </c>
       <c r="Y21" s="5" t="n">
-        <v>2243398452</v>
+        <v>2243398455</v>
       </c>
       <c r="Z21" s="5" t="inlineStr">
         <is>
@@ -4446,27 +4446,27 @@
         <v>22649882</v>
       </c>
       <c r="B22" s="5" t="n">
-        <v>23459433</v>
+        <v>23459436</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>ACC16</t>
+          <t>ACC19</t>
         </is>
       </c>
       <c r="D22" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
@@ -4481,7 +4481,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>MARIA GISANE DOS SANTOS MACHADO</t>
+          <t>HERLIA FERREIRA PEREIRA PALACIO</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -4551,7 +4551,7 @@
         </is>
       </c>
       <c r="Y22" s="5" t="n">
-        <v>2243398453</v>
+        <v>2243398456</v>
       </c>
       <c r="Z22" s="5" t="inlineStr">
         <is>
@@ -4633,27 +4633,27 @@
         <v>22649882</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>23459434</v>
+        <v>23459437</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>ACC17</t>
+          <t>ACC20</t>
         </is>
       </c>
       <c r="D23" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>RANGIELE DO CARMO ASSUNCAO</t>
+          <t>GEANNE PIRES DE MESQUITA</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
@@ -4738,7 +4738,7 @@
         </is>
       </c>
       <c r="Y23" s="5" t="n">
-        <v>2243398454</v>
+        <v>2243398457</v>
       </c>
       <c r="Z23" s="5" t="inlineStr">
         <is>
@@ -4820,27 +4820,27 @@
         <v>22649882</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>23459435</v>
+        <v>23459438</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>ACC18</t>
+          <t>ACC21</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -4855,7 +4855,7 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>LUNARA SOUSA MOTA</t>
+          <t>DANIELE FREITAS CAVALCANTE DE OLIVEIRA</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -4925,7 +4925,7 @@
         </is>
       </c>
       <c r="Y24" s="5" t="n">
-        <v>2243398455</v>
+        <v>2243398493</v>
       </c>
       <c r="Z24" s="5" t="inlineStr">
         <is>
@@ -5007,27 +5007,27 @@
         <v>22649882</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>23459436</v>
+        <v>23459439</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>ACC19</t>
+          <t>ACC22</t>
         </is>
       </c>
       <c r="D25" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>HERLIA FERREIRA PEREIRA PALACIO</t>
+          <t>ADAILMA MENDES DOS SANTOS</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="Y25" s="5" t="n">
-        <v>2243398456</v>
+        <v>2243398459</v>
       </c>
       <c r="Z25" s="5" t="inlineStr">
         <is>
@@ -5194,27 +5194,27 @@
         <v>22649882</v>
       </c>
       <c r="B26" s="5" t="n">
-        <v>23459437</v>
+        <v>23459440</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>ACC20</t>
+          <t>ACC23</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -5229,7 +5229,7 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>GEANNE PIRES DE MESQUITA</t>
+          <t>KELEN CRISTINA MARTINS ALENCAR PINTO</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -5299,7 +5299,7 @@
         </is>
       </c>
       <c r="Y26" s="5" t="n">
-        <v>2243398457</v>
+        <v>2243398460</v>
       </c>
       <c r="Z26" s="5" t="inlineStr">
         <is>
@@ -5381,27 +5381,27 @@
         <v>22649882</v>
       </c>
       <c r="B27" s="5" t="n">
-        <v>23459438</v>
+        <v>23459441</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>ACC21</t>
+          <t>ACC24</t>
         </is>
       </c>
       <c r="D27" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -5416,7 +5416,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>DANIELE FREITAS CAVALCANTE DE OLIVEIRA</t>
+          <t>JORGEANA MORAIS MONTEIRO</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
@@ -5486,7 +5486,7 @@
         </is>
       </c>
       <c r="Y27" s="5" t="n">
-        <v>2243398493</v>
+        <v>2243398461</v>
       </c>
       <c r="Z27" s="5" t="inlineStr">
         <is>
@@ -5568,27 +5568,27 @@
         <v>22649882</v>
       </c>
       <c r="B28" s="5" t="n">
-        <v>23459439</v>
+        <v>23459442</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>ACC22</t>
+          <t>ACC25</t>
         </is>
       </c>
       <c r="D28" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>ADAILMA MENDES DOS SANTOS</t>
+          <t>ANA CAROLINA CORREA</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -5673,7 +5673,7 @@
         </is>
       </c>
       <c r="Y28" s="5" t="n">
-        <v>2243398459</v>
+        <v>2243398462</v>
       </c>
       <c r="Z28" s="5" t="inlineStr">
         <is>
@@ -5755,27 +5755,27 @@
         <v>22649882</v>
       </c>
       <c r="B29" s="5" t="n">
-        <v>23459440</v>
+        <v>23459443</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>ACC23</t>
+          <t>ACC26</t>
         </is>
       </c>
       <c r="D29" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -5790,7 +5790,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>KELEN CRISTINA MARTINS ALENCAR PINTO</t>
+          <t>IRLA GOMES DE SOUZA</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -5860,7 +5860,7 @@
         </is>
       </c>
       <c r="Y29" s="5" t="n">
-        <v>2243398460</v>
+        <v>2243398463</v>
       </c>
       <c r="Z29" s="5" t="inlineStr">
         <is>
@@ -5942,27 +5942,27 @@
         <v>22649882</v>
       </c>
       <c r="B30" s="5" t="n">
-        <v>23459441</v>
+        <v>23459444</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>ACC24</t>
+          <t>ACC27</t>
         </is>
       </c>
       <c r="D30" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -5977,7 +5977,7 @@
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>JORGEANA MORAIS MONTEIRO</t>
+          <t>DAIANA MAGALHAES DE PAIVA</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -6047,7 +6047,7 @@
         </is>
       </c>
       <c r="Y30" s="5" t="n">
-        <v>2243398461</v>
+        <v>2243398464</v>
       </c>
       <c r="Z30" s="5" t="inlineStr">
         <is>
@@ -6129,27 +6129,27 @@
         <v>22649882</v>
       </c>
       <c r="B31" s="5" t="n">
-        <v>23459442</v>
+        <v>23459445</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>ACC25</t>
+          <t>ACC28</t>
         </is>
       </c>
       <c r="D31" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>ANA CAROLINA CORREA</t>
+          <t>FERNANDA HELENA ALVES DA ROCHA</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
@@ -6234,7 +6234,7 @@
         </is>
       </c>
       <c r="Y31" s="5" t="n">
-        <v>2243398462</v>
+        <v>2243398465</v>
       </c>
       <c r="Z31" s="5" t="inlineStr">
         <is>
@@ -6316,27 +6316,27 @@
         <v>22649882</v>
       </c>
       <c r="B32" s="5" t="n">
-        <v>23459443</v>
+        <v>23459446</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>ACC26</t>
+          <t>ACC29</t>
         </is>
       </c>
       <c r="D32" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>IRLA GOMES DE SOUZA</t>
+          <t>KESSYA CARDOSO LIMA</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -6421,7 +6421,7 @@
         </is>
       </c>
       <c r="Y32" s="5" t="n">
-        <v>2243398463</v>
+        <v>2243398466</v>
       </c>
       <c r="Z32" s="5" t="inlineStr">
         <is>
@@ -6503,27 +6503,27 @@
         <v>22649882</v>
       </c>
       <c r="B33" s="5" t="n">
-        <v>23459444</v>
+        <v>23459447</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>ACC27</t>
+          <t>ACC30</t>
         </is>
       </c>
       <c r="D33" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
@@ -6538,7 +6538,7 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>DAIANA MAGALHAES DE PAIVA</t>
+          <t>JESSICA CORREIA SALES</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
@@ -6608,7 +6608,7 @@
         </is>
       </c>
       <c r="Y33" s="5" t="n">
-        <v>2243398464</v>
+        <v>2243398467</v>
       </c>
       <c r="Z33" s="5" t="inlineStr">
         <is>
@@ -6690,27 +6690,27 @@
         <v>22649882</v>
       </c>
       <c r="B34" s="5" t="n">
-        <v>23459445</v>
+        <v>23459448</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>ACC28</t>
+          <t>ACC31</t>
         </is>
       </c>
       <c r="D34" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>FERNANDA HELENA ALVES DA ROCHA</t>
+          <t>MICHELLE PEREIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
@@ -6795,7 +6795,7 @@
         </is>
       </c>
       <c r="Y34" s="5" t="n">
-        <v>2243398465</v>
+        <v>2243398468</v>
       </c>
       <c r="Z34" s="5" t="inlineStr">
         <is>
@@ -6877,27 +6877,27 @@
         <v>22649882</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>23459446</v>
+        <v>23459449</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>ACC29</t>
+          <t>ACC32</t>
         </is>
       </c>
       <c r="D35" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -6912,7 +6912,7 @@
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>KESSYA CARDOSO LIMA</t>
+          <t>NATALIA TAVARES DE ALMEIDA</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
@@ -6982,7 +6982,7 @@
         </is>
       </c>
       <c r="Y35" s="5" t="n">
-        <v>2243398466</v>
+        <v>2243398469</v>
       </c>
       <c r="Z35" s="5" t="inlineStr">
         <is>
@@ -7064,27 +7064,27 @@
         <v>22649882</v>
       </c>
       <c r="B36" s="5" t="n">
-        <v>23459447</v>
+        <v>23459450</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>ACC30</t>
+          <t>ACC33</t>
         </is>
       </c>
       <c r="D36" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
@@ -7099,7 +7099,7 @@
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>JESSICA CORREIA SALES</t>
+          <t>ANDREZZA RAYANNE ALVES DE ALMEIDA</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
@@ -7169,7 +7169,7 @@
         </is>
       </c>
       <c r="Y36" s="5" t="n">
-        <v>2243398467</v>
+        <v>2243398470</v>
       </c>
       <c r="Z36" s="5" t="inlineStr">
         <is>
@@ -7251,27 +7251,27 @@
         <v>22649882</v>
       </c>
       <c r="B37" s="5" t="n">
-        <v>23459448</v>
+        <v>23459451</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>ACC31</t>
+          <t>ACC34</t>
         </is>
       </c>
       <c r="D37" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>MICHELLE PEREIRA DE OLIVEIRA</t>
+          <t>LILIAN KESSIA ALVES SIEBRA</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
@@ -7356,7 +7356,7 @@
         </is>
       </c>
       <c r="Y37" s="5" t="n">
-        <v>2243398468</v>
+        <v>2243398471</v>
       </c>
       <c r="Z37" s="5" t="inlineStr">
         <is>
@@ -7438,27 +7438,27 @@
         <v>22649882</v>
       </c>
       <c r="B38" s="5" t="n">
-        <v>23459449</v>
+        <v>23459452</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>ACC32</t>
+          <t>ACC35</t>
         </is>
       </c>
       <c r="D38" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>NATALIA TAVARES DE ALMEIDA</t>
+          <t>MONALISA DO NASCIMENTO RIBEIRO</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
@@ -7543,7 +7543,7 @@
         </is>
       </c>
       <c r="Y38" s="5" t="n">
-        <v>2243398469</v>
+        <v>2243398472</v>
       </c>
       <c r="Z38" s="5" t="inlineStr">
         <is>
@@ -7625,27 +7625,27 @@
         <v>22649882</v>
       </c>
       <c r="B39" s="5" t="n">
-        <v>23459450</v>
+        <v>23459453</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>ACC33</t>
+          <t>ACC36</t>
         </is>
       </c>
       <c r="D39" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
@@ -7660,7 +7660,7 @@
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>ANDREZZA RAYANNE ALVES DE ALMEIDA</t>
+          <t>PRISCILA ADRIAN RODRIGUES</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
@@ -7730,7 +7730,7 @@
         </is>
       </c>
       <c r="Y39" s="5" t="n">
-        <v>2243398470</v>
+        <v>2243398473</v>
       </c>
       <c r="Z39" s="5" t="inlineStr">
         <is>
@@ -7812,27 +7812,27 @@
         <v>22649882</v>
       </c>
       <c r="B40" s="5" t="n">
-        <v>23459451</v>
+        <v>23459454</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>ACC34</t>
+          <t>ACC37</t>
         </is>
       </c>
       <c r="D40" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
@@ -7847,7 +7847,7 @@
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>LILIAN KESSIA ALVES SIEBRA</t>
+          <t>NATALIA FARIAS DE SOUSA</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
@@ -7917,7 +7917,7 @@
         </is>
       </c>
       <c r="Y40" s="5" t="n">
-        <v>2243398471</v>
+        <v>2243398474</v>
       </c>
       <c r="Z40" s="5" t="inlineStr">
         <is>
@@ -7999,27 +7999,27 @@
         <v>22649882</v>
       </c>
       <c r="B41" s="5" t="n">
-        <v>23459452</v>
+        <v>23459455</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>ACC35</t>
+          <t>ACC38</t>
         </is>
       </c>
       <c r="D41" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E41" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>MONALISA DO NASCIMENTO RIBEIRO</t>
+          <t>MARIANA MELO CAMURCA</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
@@ -8104,7 +8104,7 @@
         </is>
       </c>
       <c r="Y41" s="5" t="n">
-        <v>2243398472</v>
+        <v>2243398475</v>
       </c>
       <c r="Z41" s="5" t="inlineStr">
         <is>
@@ -8186,27 +8186,27 @@
         <v>22649882</v>
       </c>
       <c r="B42" s="5" t="n">
-        <v>23459453</v>
+        <v>23459456</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>ACC36</t>
+          <t>ACC39</t>
         </is>
       </c>
       <c r="D42" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
@@ -8221,7 +8221,7 @@
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>PRISCILA ADRIAN RODRIGUES</t>
+          <t>YOHANNA MARIA MENEZES DO NASCIMENTO</t>
         </is>
       </c>
       <c r="K42" s="5" t="inlineStr">
@@ -8291,7 +8291,7 @@
         </is>
       </c>
       <c r="Y42" s="5" t="n">
-        <v>2243398473</v>
+        <v>2243398476</v>
       </c>
       <c r="Z42" s="5" t="inlineStr">
         <is>
@@ -8373,27 +8373,27 @@
         <v>22649882</v>
       </c>
       <c r="B43" s="5" t="n">
-        <v>23459454</v>
+        <v>23459457</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>ACC37</t>
+          <t>ACC40</t>
         </is>
       </c>
       <c r="D43" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>NATALIA FARIAS DE SOUSA</t>
+          <t>MARIA ELINARA COSTA REBOUCAS</t>
         </is>
       </c>
       <c r="K43" s="5" t="inlineStr">
@@ -8478,7 +8478,7 @@
         </is>
       </c>
       <c r="Y43" s="5" t="n">
-        <v>2243398474</v>
+        <v>2243398477</v>
       </c>
       <c r="Z43" s="5" t="inlineStr">
         <is>
@@ -8560,27 +8560,27 @@
         <v>22649882</v>
       </c>
       <c r="B44" s="5" t="n">
-        <v>23459455</v>
+        <v>23459458</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>ACC38</t>
+          <t>ACC41</t>
         </is>
       </c>
       <c r="D44" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
@@ -8595,7 +8595,7 @@
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>MARIANA MELO CAMURCA</t>
+          <t>ANA MICHELLE LOUREIRO LOBO</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="Y44" s="5" t="n">
-        <v>2243398475</v>
+        <v>2243398478</v>
       </c>
       <c r="Z44" s="5" t="inlineStr">
         <is>
@@ -8747,27 +8747,27 @@
         <v>22649882</v>
       </c>
       <c r="B45" s="5" t="n">
-        <v>23459456</v>
+        <v>23459459</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>ACC39</t>
+          <t>ACC42</t>
         </is>
       </c>
       <c r="D45" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
@@ -8782,7 +8782,7 @@
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>YOHANNA MARIA MENEZES DO NASCIMENTO</t>
+          <t>MAIARA MARIA NASCIMENTO DE ARAUJO</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">
@@ -8852,7 +8852,7 @@
         </is>
       </c>
       <c r="Y45" s="5" t="n">
-        <v>2243398476</v>
+        <v>2243398479</v>
       </c>
       <c r="Z45" s="5" t="inlineStr">
         <is>
@@ -8934,27 +8934,27 @@
         <v>22649882</v>
       </c>
       <c r="B46" s="5" t="n">
-        <v>23459457</v>
+        <v>23459460</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>ACC40</t>
+          <t>ACC43</t>
         </is>
       </c>
       <c r="D46" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
@@ -8969,7 +8969,7 @@
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>MARIA ELINARA COSTA REBOUCAS</t>
+          <t>THISIANIA ROMERO VIEIRA SOARES</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
@@ -9039,7 +9039,7 @@
         </is>
       </c>
       <c r="Y46" s="5" t="n">
-        <v>2243398477</v>
+        <v>2243398480</v>
       </c>
       <c r="Z46" s="5" t="inlineStr">
         <is>
@@ -9121,27 +9121,27 @@
         <v>22649882</v>
       </c>
       <c r="B47" s="5" t="n">
-        <v>23459458</v>
+        <v>23459461</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>ACC41</t>
+          <t>ACC44</t>
         </is>
       </c>
       <c r="D47" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
@@ -9156,7 +9156,7 @@
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>ANA MICHELLE LOUREIRO LOBO</t>
+          <t>CRISLANE ALENCARINA LIMA DA SILVA</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
@@ -9226,7 +9226,7 @@
         </is>
       </c>
       <c r="Y47" s="5" t="n">
-        <v>2243398478</v>
+        <v>2243398481</v>
       </c>
       <c r="Z47" s="5" t="inlineStr">
         <is>
@@ -9308,27 +9308,27 @@
         <v>22649882</v>
       </c>
       <c r="B48" s="5" t="n">
-        <v>23459459</v>
+        <v>23459462</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>ACC42</t>
+          <t>ACC45</t>
         </is>
       </c>
       <c r="D48" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
@@ -9343,7 +9343,7 @@
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>MAIARA MARIA NASCIMENTO DE ARAUJO</t>
+          <t>PAULA AMANDA DO CARMO FERNANDES</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">
@@ -9413,7 +9413,7 @@
         </is>
       </c>
       <c r="Y48" s="5" t="n">
-        <v>2243398479</v>
+        <v>2243398482</v>
       </c>
       <c r="Z48" s="5" t="inlineStr">
         <is>
@@ -9495,27 +9495,27 @@
         <v>22649882</v>
       </c>
       <c r="B49" s="5" t="n">
-        <v>23459460</v>
+        <v>23459463</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>ACC43</t>
+          <t>ACC46</t>
         </is>
       </c>
       <c r="D49" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
@@ -9530,7 +9530,7 @@
       </c>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>THISIANIA ROMERO VIEIRA SOARES</t>
+          <t>DIANA CARLA MORAES DOS SANTOS</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr">
@@ -9600,7 +9600,7 @@
         </is>
       </c>
       <c r="Y49" s="5" t="n">
-        <v>2243398480</v>
+        <v>2243398483</v>
       </c>
       <c r="Z49" s="5" t="inlineStr">
         <is>
@@ -9682,27 +9682,27 @@
         <v>22649882</v>
       </c>
       <c r="B50" s="5" t="n">
-        <v>23459461</v>
+        <v>23459465</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>ACC44</t>
+          <t>ACC47</t>
         </is>
       </c>
       <c r="D50" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
@@ -9717,7 +9717,7 @@
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>CRISLANE ALENCARINA LIMA DA SILVA</t>
+          <t>LUDMILA VIRNA OLIVEIRA FERNANDES</t>
         </is>
       </c>
       <c r="K50" s="5" t="inlineStr">
@@ -9787,7 +9787,7 @@
         </is>
       </c>
       <c r="Y50" s="5" t="n">
-        <v>2243398481</v>
+        <v>2243398484</v>
       </c>
       <c r="Z50" s="5" t="inlineStr">
         <is>
@@ -9869,27 +9869,27 @@
         <v>22649882</v>
       </c>
       <c r="B51" s="5" t="n">
-        <v>23459462</v>
+        <v>23459466</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>ACC45</t>
+          <t>ACC48</t>
         </is>
       </c>
       <c r="D51" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
@@ -9904,7 +9904,7 @@
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>PAULA AMANDA DO CARMO FERNANDES</t>
+          <t>CLAUDIANA HONORATO MIGUEL</t>
         </is>
       </c>
       <c r="K51" s="5" t="inlineStr">
@@ -9974,7 +9974,7 @@
         </is>
       </c>
       <c r="Y51" s="5" t="n">
-        <v>2243398482</v>
+        <v>2243398485</v>
       </c>
       <c r="Z51" s="5" t="inlineStr">
         <is>
@@ -10056,27 +10056,27 @@
         <v>22649882</v>
       </c>
       <c r="B52" s="5" t="n">
-        <v>23459463</v>
+        <v>23459467</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>ACC46</t>
+          <t>ACC49</t>
         </is>
       </c>
       <c r="D52" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
@@ -10091,7 +10091,7 @@
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>DIANA CARLA MORAES DOS SANTOS</t>
+          <t>SAN MILK RODRIGUES QUEIROZ</t>
         </is>
       </c>
       <c r="K52" s="5" t="inlineStr">
@@ -10161,7 +10161,7 @@
         </is>
       </c>
       <c r="Y52" s="5" t="n">
-        <v>2243398483</v>
+        <v>2243398486</v>
       </c>
       <c r="Z52" s="5" t="inlineStr">
         <is>
@@ -10243,27 +10243,27 @@
         <v>22649882</v>
       </c>
       <c r="B53" s="5" t="n">
-        <v>23459465</v>
+        <v>23459468</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>ACC47</t>
+          <t>ACC50</t>
         </is>
       </c>
       <c r="D53" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
@@ -10278,7 +10278,7 @@
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>LUDMILA VIRNA OLIVEIRA FERNANDES</t>
+          <t>JENNIFER MAINARA DA SILVA FACANHA</t>
         </is>
       </c>
       <c r="K53" s="5" t="inlineStr">
@@ -10348,7 +10348,7 @@
         </is>
       </c>
       <c r="Y53" s="5" t="n">
-        <v>2243398484</v>
+        <v>2243398487</v>
       </c>
       <c r="Z53" s="5" t="inlineStr">
         <is>
@@ -10430,27 +10430,27 @@
         <v>22649882</v>
       </c>
       <c r="B54" s="5" t="n">
-        <v>23459466</v>
+        <v>23459469</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>ACC48</t>
+          <t>ACC51</t>
         </is>
       </c>
       <c r="D54" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
@@ -10465,7 +10465,7 @@
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>CLAUDIANA HONORATO MIGUEL</t>
+          <t>THAIS MESQUITA GARCIA</t>
         </is>
       </c>
       <c r="K54" s="5" t="inlineStr">
@@ -10535,7 +10535,7 @@
         </is>
       </c>
       <c r="Y54" s="5" t="n">
-        <v>2243398485</v>
+        <v>2243398488</v>
       </c>
       <c r="Z54" s="5" t="inlineStr">
         <is>
@@ -10617,27 +10617,27 @@
         <v>22649882</v>
       </c>
       <c r="B55" s="5" t="n">
-        <v>23459467</v>
+        <v>23459470</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>ACC49</t>
+          <t>ACC52</t>
         </is>
       </c>
       <c r="D55" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
@@ -10652,7 +10652,7 @@
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>SAN MILK RODRIGUES QUEIROZ</t>
+          <t>ARLETE CAVALCANTE ASSUNCAO</t>
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr">
@@ -10722,7 +10722,7 @@
         </is>
       </c>
       <c r="Y55" s="5" t="n">
-        <v>2243398486</v>
+        <v>2243398489</v>
       </c>
       <c r="Z55" s="5" t="inlineStr">
         <is>
@@ -10804,27 +10804,27 @@
         <v>22649882</v>
       </c>
       <c r="B56" s="5" t="n">
-        <v>23459468</v>
+        <v>23459471</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>ACC50</t>
+          <t>ACC53</t>
         </is>
       </c>
       <c r="D56" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>JENNIFER MAINARA DA SILVA FACANHA</t>
+          <t>KELIANE DA SILVA SOARES</t>
         </is>
       </c>
       <c r="K56" s="5" t="inlineStr">
@@ -10909,7 +10909,7 @@
         </is>
       </c>
       <c r="Y56" s="5" t="n">
-        <v>2243398487</v>
+        <v>2243398490</v>
       </c>
       <c r="Z56" s="5" t="inlineStr">
         <is>
@@ -10991,27 +10991,27 @@
         <v>22649882</v>
       </c>
       <c r="B57" s="5" t="n">
-        <v>23459469</v>
+        <v>23459472</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>ACC51</t>
+          <t>ACC54</t>
         </is>
       </c>
       <c r="D57" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
@@ -11026,7 +11026,7 @@
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>THAIS MESQUITA GARCIA</t>
+          <t>MIKAELLA DOS SANTOS ALVES</t>
         </is>
       </c>
       <c r="K57" s="5" t="inlineStr">
@@ -11096,7 +11096,7 @@
         </is>
       </c>
       <c r="Y57" s="5" t="n">
-        <v>2243398488</v>
+        <v>2243398491</v>
       </c>
       <c r="Z57" s="5" t="inlineStr">
         <is>
@@ -11178,27 +11178,27 @@
         <v>22649882</v>
       </c>
       <c r="B58" s="5" t="n">
-        <v>23459470</v>
+        <v>23459473</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>ACC52</t>
+          <t>ACC55</t>
         </is>
       </c>
       <c r="D58" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr">
@@ -11213,7 +11213,7 @@
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>ARLETE CAVALCANTE ASSUNCAO</t>
+          <t>ANNA CLARA DOMINGOS ALVES</t>
         </is>
       </c>
       <c r="K58" s="5" t="inlineStr">
@@ -11283,7 +11283,7 @@
         </is>
       </c>
       <c r="Y58" s="5" t="n">
-        <v>2243398489</v>
+        <v>2243398492</v>
       </c>
       <c r="Z58" s="5" t="inlineStr">
         <is>
@@ -11365,27 +11365,27 @@
         <v>22649882</v>
       </c>
       <c r="B59" s="5" t="n">
-        <v>23459471</v>
+        <v>23459474</v>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>ACC53</t>
+          <t>ACC56</t>
         </is>
       </c>
       <c r="D59" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr">
@@ -11400,7 +11400,7 @@
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>KELIANE DA SILVA SOARES</t>
+          <t>FRANCISCA ERICA COSTA DE MENEZES</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
@@ -11470,7 +11470,7 @@
         </is>
       </c>
       <c r="Y59" s="5" t="n">
-        <v>2243398490</v>
+        <v>2243398493</v>
       </c>
       <c r="Z59" s="5" t="inlineStr">
         <is>
@@ -11552,27 +11552,27 @@
         <v>22649882</v>
       </c>
       <c r="B60" s="5" t="n">
-        <v>23459472</v>
+        <v>23459475</v>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>ACC54</t>
+          <t>ACC57</t>
         </is>
       </c>
       <c r="D60" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
@@ -11587,7 +11587,7 @@
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>MIKAELLA DOS SANTOS ALVES</t>
+          <t>LUIZIANNE MARIA GONCALVES DE ALENCAR</t>
         </is>
       </c>
       <c r="K60" s="5" t="inlineStr">
@@ -11657,7 +11657,7 @@
         </is>
       </c>
       <c r="Y60" s="5" t="n">
-        <v>2243398491</v>
+        <v>2243398494</v>
       </c>
       <c r="Z60" s="5" t="inlineStr">
         <is>
@@ -11739,27 +11739,27 @@
         <v>22649882</v>
       </c>
       <c r="B61" s="5" t="n">
-        <v>23459473</v>
+        <v>23459476</v>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>ACC55</t>
+          <t>ACC58</t>
         </is>
       </c>
       <c r="D61" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E61" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
@@ -11774,7 +11774,7 @@
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>ANNA CLARA DOMINGOS ALVES</t>
+          <t>LUAN MIKAEL DE SOUSA PEREIRA</t>
         </is>
       </c>
       <c r="K61" s="5" t="inlineStr">
@@ -11844,7 +11844,7 @@
         </is>
       </c>
       <c r="Y61" s="5" t="n">
-        <v>2243398492</v>
+        <v>2243398495</v>
       </c>
       <c r="Z61" s="5" t="inlineStr">
         <is>
@@ -11926,27 +11926,27 @@
         <v>22649882</v>
       </c>
       <c r="B62" s="5" t="n">
-        <v>23459474</v>
+        <v>23459477</v>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>ACC56</t>
+          <t>ACC59</t>
         </is>
       </c>
       <c r="D62" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
@@ -11961,7 +11961,7 @@
       </c>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>FRANCISCA ERICA COSTA DE MENEZES</t>
+          <t>ANA CAROLINA MOREIRA QUEIROZ</t>
         </is>
       </c>
       <c r="K62" s="5" t="inlineStr">
@@ -12031,7 +12031,7 @@
         </is>
       </c>
       <c r="Y62" s="5" t="n">
-        <v>2243398493</v>
+        <v>2243398496</v>
       </c>
       <c r="Z62" s="5" t="inlineStr">
         <is>
@@ -12113,27 +12113,27 @@
         <v>22649882</v>
       </c>
       <c r="B63" s="5" t="n">
-        <v>23459475</v>
+        <v>23459478</v>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>ACC57</t>
+          <t>ACC60</t>
         </is>
       </c>
       <c r="D63" s="6" t="n">
         <v>45868.40885416666</v>
       </c>
       <c r="E63" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.85440972223</v>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr">
@@ -12148,7 +12148,7 @@
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>LUIZIANNE MARIA GONCALVES DE ALENCAR</t>
+          <t>GABRIEL DA SILVA ROCHA</t>
         </is>
       </c>
       <c r="K63" s="5" t="inlineStr">
@@ -12218,7 +12218,7 @@
         </is>
       </c>
       <c r="Y63" s="5" t="n">
-        <v>2243398494</v>
+        <v>2243398497</v>
       </c>
       <c r="Z63" s="5" t="inlineStr">
         <is>
@@ -12297,35 +12297,35 @@
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
-        <v>22649882</v>
+        <v>22679559</v>
       </c>
       <c r="B64" s="5" t="n">
-        <v>23459476</v>
+        <v>23484064</v>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>ACC58</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D64" s="6" t="n">
-        <v>45868.40885416666</v>
+        <v>45873.65900462963</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.64171296296</v>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr">
         <is>
-          <t>HNMBIK</t>
+          <t>B3NZNT</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
@@ -12335,24 +12335,26 @@
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>LUAN MIKAEL DE SOUSA PEREIRA</t>
+          <t>BUENO BARBOSA/RENATA</t>
         </is>
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t>Jaqueline Rodrigues Teixeira</t>
+          <t>Danny Junqueira Martins</t>
         </is>
       </c>
       <c r="L64" s="5" t="inlineStr">
         <is>
-          <t>Jaqueline Rodrigues Teixeira</t>
+          <t>Danny Junqueira Martins</t>
         </is>
       </c>
       <c r="M64" s="6" t="n">
-        <v>45867</v>
-      </c>
-      <c r="N64" s="5" t="n">
-        <v>4801518571</v>
+        <v>45873.65833333333</v>
+      </c>
+      <c r="N64" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O64" s="5" t="inlineStr">
         <is>
@@ -12386,46 +12388,48 @@
       </c>
       <c r="U64" s="5" t="inlineStr">
         <is>
-          <t>Grupo Diageo</t>
+          <t>Grupo Jti</t>
         </is>
       </c>
       <c r="V64" s="5" t="inlineStr">
         <is>
-          <t>Diageo Brasil</t>
+          <t>Jti Distribuidora - Sao Paulo - Vila Nova Conceicao</t>
         </is>
       </c>
       <c r="W64" s="5" t="inlineStr">
         <is>
-          <t>Cliente FEE no POS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="X64" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="Y64" s="5" t="n">
-        <v>2243398495</v>
+        <v>2971556787</v>
       </c>
       <c r="Z64" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>
       </c>
-      <c r="AA64" s="5" t="n">
-        <v>167526</v>
+      <c r="AA64" s="5" t="inlineStr">
+        <is>
+          <t>ID152723</t>
+        </is>
       </c>
       <c r="AB64" s="5" t="n">
-        <v>683.05</v>
+        <v>6420.23</v>
       </c>
       <c r="AC64" s="5" t="n">
-        <v>31.44</v>
+        <v>464.43</v>
       </c>
       <c r="AD64" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE64" s="5" t="n">
-        <v>68.25</v>
+        <v>0</v>
       </c>
       <c r="AF64" s="5" t="n">
         <v>0</v>
@@ -12434,16 +12438,16 @@
         <v>0</v>
       </c>
       <c r="AH64" s="5" t="n">
-        <v>86.09999999999999</v>
+        <v>655.21</v>
       </c>
       <c r="AI64" s="5" t="inlineStr">
         <is>
-          <t>Reserva importada via planilha. Solicitação: |PC:</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AJ64" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2243398493 já sendo utilizado para este fornecedor.</t>
+          <t>Verificação de bilhetes: Bilhete 2971556787 já sendo utilizado para este fornecedor.</t>
         </is>
       </c>
       <c r="AK64" s="5" t="inlineStr">
@@ -12484,35 +12488,35 @@
     </row>
     <row r="65">
       <c r="A65" s="5" t="n">
-        <v>22649882</v>
+        <v>22679559</v>
       </c>
       <c r="B65" s="5" t="n">
-        <v>23459477</v>
+        <v>23484078</v>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>ACC59</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D65" s="6" t="n">
-        <v>45868.40885416666</v>
+        <v>45873.65900462963</v>
       </c>
       <c r="E65" s="6" t="n">
-        <v>45868.41748842593</v>
+        <v>45874.64171296296</v>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>HNMBIK</t>
+          <t>B3NZNT</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
@@ -12522,24 +12526,26 @@
       </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>ANA CAROLINA MOREIRA QUEIROZ</t>
+          <t>SIMOES BARBOSA/FRANCISCO</t>
         </is>
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
-          <t>Jaqueline Rodrigues Teixeira</t>
+          <t>Danny Junqueira Martins</t>
         </is>
       </c>
       <c r="L65" s="5" t="inlineStr">
         <is>
-          <t>Jaqueline Rodrigues Teixeira</t>
+          <t>Danny Junqueira Martins</t>
         </is>
       </c>
       <c r="M65" s="6" t="n">
-        <v>45867</v>
-      </c>
-      <c r="N65" s="5" t="n">
-        <v>4801518571</v>
+        <v>45873.65833333333</v>
+      </c>
+      <c r="N65" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O65" s="5" t="inlineStr">
         <is>
@@ -12573,46 +12579,48 @@
       </c>
       <c r="U65" s="5" t="inlineStr">
         <is>
-          <t>Grupo Diageo</t>
+          <t>Grupo Jti</t>
         </is>
       </c>
       <c r="V65" s="5" t="inlineStr">
         <is>
-          <t>Diageo Brasil</t>
+          <t>Jti Distribuidora - Sao Paulo - Vila Nova Conceicao</t>
         </is>
       </c>
       <c r="W65" s="5" t="inlineStr">
         <is>
-          <t>Cliente FEE no POS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="X65" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Iberia</t>
         </is>
       </c>
       <c r="Y65" s="5" t="n">
-        <v>2243398496</v>
+        <v>2971556785</v>
       </c>
       <c r="Z65" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>
       </c>
-      <c r="AA65" s="5" t="n">
-        <v>167526</v>
+      <c r="AA65" s="5" t="inlineStr">
+        <is>
+          <t>ID152723</t>
+        </is>
       </c>
       <c r="AB65" s="5" t="n">
-        <v>683.05</v>
+        <v>6420.23</v>
       </c>
       <c r="AC65" s="5" t="n">
-        <v>31.44</v>
+        <v>464.43</v>
       </c>
       <c r="AD65" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE65" s="5" t="n">
-        <v>68.25</v>
+        <v>0</v>
       </c>
       <c r="AF65" s="5" t="n">
         <v>0</v>
@@ -12621,16 +12629,16 @@
         <v>0</v>
       </c>
       <c r="AH65" s="5" t="n">
-        <v>86.09999999999999</v>
+        <v>655.21</v>
       </c>
       <c r="AI65" s="5" t="inlineStr">
         <is>
-          <t>Reserva importada via planilha. Solicitação: |PC:</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AJ65" s="5" t="inlineStr">
         <is>
-          <t>Verificação de bilhetes: Bilhete 2243398493 já sendo utilizado para este fornecedor.</t>
+          <t>Verificação de bilhetes: Bilhete 2971556787 já sendo utilizado para este fornecedor.</t>
         </is>
       </c>
       <c r="AK65" s="5" t="inlineStr">
@@ -12664,193 +12672,6 @@
         </is>
       </c>
       <c r="AQ65" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="n">
-        <v>22649882</v>
-      </c>
-      <c r="B66" s="5" t="n">
-        <v>23459478</v>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>ACC60</t>
-        </is>
-      </c>
-      <c r="D66" s="6" t="n">
-        <v>45868.40885416666</v>
-      </c>
-      <c r="E66" s="6" t="n">
-        <v>45868.41748842593</v>
-      </c>
-      <c r="F66" s="5" t="inlineStr">
-        <is>
-          <t>06 a 08 dias</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="inlineStr">
-        <is>
-          <t>06 a 08 dias</t>
-        </is>
-      </c>
-      <c r="H66" s="5" t="inlineStr">
-        <is>
-          <t>HNMBIK</t>
-        </is>
-      </c>
-      <c r="I66" s="5" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="J66" s="5" t="inlineStr">
-        <is>
-          <t>GABRIEL DA SILVA ROCHA</t>
-        </is>
-      </c>
-      <c r="K66" s="5" t="inlineStr">
-        <is>
-          <t>Jaqueline Rodrigues Teixeira</t>
-        </is>
-      </c>
-      <c r="L66" s="5" t="inlineStr">
-        <is>
-          <t>Jaqueline Rodrigues Teixeira</t>
-        </is>
-      </c>
-      <c r="M66" s="6" t="n">
-        <v>45867</v>
-      </c>
-      <c r="N66" s="5" t="n">
-        <v>4801518571</v>
-      </c>
-      <c r="O66" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P66" s="5" t="inlineStr">
-        <is>
-          <t>OFF LINE</t>
-        </is>
-      </c>
-      <c r="Q66" s="5" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
-      <c r="R66" s="5" t="inlineStr">
-        <is>
-          <t>Faturado</t>
-        </is>
-      </c>
-      <c r="S66" s="5" t="inlineStr">
-        <is>
-          <t>Aéreo</t>
-        </is>
-      </c>
-      <c r="T66" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="U66" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Diageo</t>
-        </is>
-      </c>
-      <c r="V66" s="5" t="inlineStr">
-        <is>
-          <t>Diageo Brasil</t>
-        </is>
-      </c>
-      <c r="W66" s="5" t="inlineStr">
-        <is>
-          <t>Cliente FEE no POS</t>
-        </is>
-      </c>
-      <c r="X66" s="5" t="inlineStr">
-        <is>
-          <t>Latam Airlines Brasil</t>
-        </is>
-      </c>
-      <c r="Y66" s="5" t="n">
-        <v>2243398497</v>
-      </c>
-      <c r="Z66" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-      <c r="AA66" s="5" t="n">
-        <v>167526</v>
-      </c>
-      <c r="AB66" s="5" t="n">
-        <v>683.05</v>
-      </c>
-      <c r="AC66" s="5" t="n">
-        <v>31.44</v>
-      </c>
-      <c r="AD66" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE66" s="5" t="n">
-        <v>68.25</v>
-      </c>
-      <c r="AF66" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG66" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH66" s="5" t="n">
-        <v>86.09999999999999</v>
-      </c>
-      <c r="AI66" s="5" t="inlineStr">
-        <is>
-          <t>Reserva importada via planilha. Solicitação: |PC:</t>
-        </is>
-      </c>
-      <c r="AJ66" s="5" t="inlineStr">
-        <is>
-          <t>Verificação de bilhetes: Bilhete 2243398493 já sendo utilizado para este fornecedor.</t>
-        </is>
-      </c>
-      <c r="AK66" s="5" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="AL66" s="5" t="inlineStr">
-        <is>
-          <t>Bilhete duplicado</t>
-        </is>
-      </c>
-      <c r="AM66" s="5" t="inlineStr">
-        <is>
-          <t>Bilhete Já Contabilizado</t>
-        </is>
-      </c>
-      <c r="AN66" s="5" t="inlineStr">
-        <is>
-          <t>Duplicidade de Contabilização</t>
-        </is>
-      </c>
-      <c r="AO66" s="5" t="inlineStr">
-        <is>
-          <t>Qualidade dos dados</t>
-        </is>
-      </c>
-      <c r="AP66" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-      <c r="AQ66" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>

</xml_diff>

<commit_message>
Update Excel reports and add new PDF reports
Updated multiple Excel files in the Integration-Quality directory, including company-specific reports and error logs. Added two new PDF reports for 15.08.2025 and 18.08.2025 to the PDFs folder.
</commit_message>
<xml_diff>
--- a/Integration-Quality/EMPRESAS/Relatorio - INOVENTS.xlsx
+++ b/Integration-Quality/EMPRESAS/Relatorio - INOVENTS.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ2"/>
+  <dimension ref="A1:AQ5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,35 +695,35 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>22728403</v>
+        <v>22746611</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>23526021</v>
+        <v>23542762</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>45881.40568287037</v>
+        <v>45884.34997685185</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>45881.41440972222</v>
+        <v>45884.35454861111</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>03 a 05 dias</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>QDSYOF</t>
+          <t>5HQ3CX</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -733,21 +733,21 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>LILIANE BARBOSA JESUS</t>
+          <t>SERVICO</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Marcelo Soares de Azevedo</t>
+          <t>Elaine Cristina Martins</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Marcelo Soares de Azevedo</t>
+          <t>Elaine Cristina Martins</t>
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>45881.40555555555</v>
+        <v>45884.34930555556</v>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
@@ -766,117 +766,692 @@
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Faturado</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>Aéreo</t>
+          <t>Serviço</t>
         </is>
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Consolidacao</t>
+        </is>
+      </c>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
+          <t>Kontik Franstur Matriz/sao Paulo</t>
+        </is>
+      </c>
+      <c r="W2" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X2" s="5" t="inlineStr">
+        <is>
+          <t>Sirena Textil</t>
+        </is>
+      </c>
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="n">
+        <v>168578</v>
+      </c>
+      <c r="AB2" s="5" t="n">
+        <v>5215.14</v>
+      </c>
+      <c r="AC2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ2" s="5" t="inlineStr">
+        <is>
+          <t>Necessário cadastrar um contrato para o cliente ""</t>
+        </is>
+      </c>
+      <c r="AK2" s="5" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="AL2" s="5" t="inlineStr">
+        <is>
+          <t>Contrato de fornecedor</t>
+        </is>
+      </c>
+      <c r="AM2" s="5" t="inlineStr">
+        <is>
+          <t>Análise Cadastro</t>
+        </is>
+      </c>
+      <c r="AN2" s="5" t="inlineStr">
+        <is>
+          <t>Dados do Fornecedor</t>
+        </is>
+      </c>
+      <c r="AO2" s="5" t="inlineStr">
+        <is>
+          <t>Qualidade dos dados</t>
+        </is>
+      </c>
+      <c r="AP2" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+      <c r="AQ2" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>22741610</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>23538473</v>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>ACC01</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>45883.51908564815</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>45884.35450231482</v>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>5HTMEQ</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>SERVICO</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Elaine Cristina Martins</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Elaine Cristina Martins</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="n">
+        <v>45883.51875</v>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>Faturado</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>Serviço</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Consolidacao</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>Kontik Franstur Matriz/sao Paulo</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>Sirena Textil</t>
+        </is>
+      </c>
+      <c r="Y3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="n">
+        <v>168578</v>
+      </c>
+      <c r="AB3" s="5" t="n">
+        <v>5215.14</v>
+      </c>
+      <c r="AC3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ3" s="5" t="inlineStr">
+        <is>
+          <t>Necessário cadastrar um contrato para o cliente ""</t>
+        </is>
+      </c>
+      <c r="AK3" s="5" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="AL3" s="5" t="inlineStr">
+        <is>
+          <t>Contrato de fornecedor</t>
+        </is>
+      </c>
+      <c r="AM3" s="5" t="inlineStr">
+        <is>
+          <t>Análise Cadastro</t>
+        </is>
+      </c>
+      <c r="AN3" s="5" t="inlineStr">
+        <is>
+          <t>Dados do Fornecedor</t>
+        </is>
+      </c>
+      <c r="AO3" s="5" t="inlineStr">
+        <is>
+          <t>Qualidade dos dados</t>
+        </is>
+      </c>
+      <c r="AP3" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+      <c r="AQ3" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>22749021</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>23544966</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>ACC01</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>45884.61769675926</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>45884.61927083333</v>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">165858-414749-B </t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> HOSPEDAGEM EM SANTA RITA DO SAPUCAÍ</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Caio Jose Albuquerque Santos</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Caio Jose Albuquerque Santos</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="n">
+        <v>45884.61736111111</v>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>Faturado</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U2" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Vertex</t>
-        </is>
-      </c>
-      <c r="V2" s="5" t="inlineStr">
-        <is>
-          <t>Vertex Farmaceutica do Brasil</t>
-        </is>
-      </c>
-      <c r="W2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X2" s="5" t="inlineStr">
-        <is>
-          <t>Latam Airlines Brasil</t>
-        </is>
-      </c>
-      <c r="Y2" s="5" t="n">
-        <v>2952818682</v>
-      </c>
-      <c r="Z2" s="5" t="inlineStr">
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Claro Sa</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
+          <t>Claro Sao Paulo (santo Amaro)</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X4" s="5" t="inlineStr">
+        <is>
+          <t>Hotel Amantykir</t>
+        </is>
+      </c>
+      <c r="Y4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z4" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>
       </c>
-      <c r="AA2" s="5" t="n">
-        <v>169348</v>
-      </c>
-      <c r="AB2" s="5" t="n">
-        <v>3472.02</v>
-      </c>
-      <c r="AC2" s="5" t="n">
-        <v>81.08</v>
-      </c>
-      <c r="AD2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="5" t="n">
-        <v>347.2</v>
-      </c>
-      <c r="AF2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH2" s="5" t="n">
-        <v>54.72</v>
-      </c>
-      <c r="AI2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ2" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ocorreu a seguinte exceção ao gerar a ordem de venda para a accounting: Ocorreu a seguinte exceção ao inserir o item da ordem de venda:  Faltou </t>
-        </is>
-      </c>
-      <c r="AK2" s="5" t="inlineStr">
+      <c r="AA4" s="5" t="n">
+        <v>165858</v>
+      </c>
+      <c r="AB4" s="5" t="n">
+        <v>12852</v>
+      </c>
+      <c r="AC4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="5" t="n">
+        <v>642.6</v>
+      </c>
+      <c r="AH4" s="5" t="n">
+        <v>2053.6</v>
+      </c>
+      <c r="AI4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> HOSPEDAGEM EM SANTA RITA DO SAPUCAÍ</t>
+        </is>
+      </c>
+      <c r="AJ4" s="5" t="inlineStr">
+        <is>
+          <t>Centro de custo não preenchido! (ACC01)</t>
+        </is>
+      </c>
+      <c r="AK4" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="AL4" s="5" t="inlineStr">
+        <is>
+          <t>Centro de custo</t>
+        </is>
+      </c>
+      <c r="AM4" s="5" t="inlineStr">
+        <is>
+          <t>Falta de informação Gerencial</t>
+        </is>
+      </c>
+      <c r="AN4" s="5" t="inlineStr">
+        <is>
+          <t>Dados do Fornecedor</t>
+        </is>
+      </c>
+      <c r="AO4" s="5" t="inlineStr">
+        <is>
+          <t>Qualidade dos dados</t>
+        </is>
+      </c>
+      <c r="AP4" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+      <c r="AQ4" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>22749395</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>23545373</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>ACC01</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>45884.66975694444</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>45884.67158564815</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>03 a 05 dias</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>5H2OKX</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="AL2" s="5" t="inlineStr">
-        <is>
-          <t>Falta de informação Gerencial</t>
-        </is>
-      </c>
-      <c r="AM2" s="5" t="inlineStr">
-        <is>
-          <t>Rateio de centro de custo/projeto</t>
-        </is>
-      </c>
-      <c r="AN2" s="5" t="inlineStr">
-        <is>
-          <t>Dados Gerenciais</t>
-        </is>
-      </c>
-      <c r="AO2" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>SERVICO</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Elaine Cristina Martins</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Elaine Cristina Martins</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>45884.66944444444</v>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>Faturado</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>Serviço</t>
+        </is>
+      </c>
+      <c r="T5" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Consolidacao</t>
+        </is>
+      </c>
+      <c r="V5" s="5" t="inlineStr">
+        <is>
+          <t>Kontik Franstur Matriz/sao Paulo</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X5" s="5" t="inlineStr">
+        <is>
+          <t>Sirena Textil</t>
+        </is>
+      </c>
+      <c r="Y5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z5" s="5" t="inlineStr">
+        <is>
+          <t>INOVENTS</t>
+        </is>
+      </c>
+      <c r="AA5" s="5" t="n">
+        <v>168578</v>
+      </c>
+      <c r="AB5" s="5" t="n">
+        <v>5215.14</v>
+      </c>
+      <c r="AC5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ5" s="5" t="inlineStr">
+        <is>
+          <t>Necessário informar a filial do cliente "Kontik Franstur Matriz/sao Paulo" em seu contrato</t>
+        </is>
+      </c>
+      <c r="AK5" s="5" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="AL5" s="5" t="inlineStr">
+        <is>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="AM5" s="5" t="inlineStr">
+        <is>
+          <t>Análise Benner</t>
+        </is>
+      </c>
+      <c r="AN5" s="5" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="AO5" s="5" t="inlineStr">
         <is>
           <t>Qualidade dos dados</t>
         </is>
       </c>
-      <c r="AP2" s="5" t="inlineStr">
+      <c r="AP5" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>
       </c>
-      <c r="AQ2" s="5" t="inlineStr">
+      <c r="AQ5" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>

</xml_diff>

<commit_message>
Update reports and add new PDF summaries
Updated multiple Excel and Power BI report files across the Integration-Quality directory. Added new PDF summary reports for dates 19.08.2025 to 22.08.2025 in the PDFs folder.
</commit_message>
<xml_diff>
--- a/Integration-Quality/EMPRESAS/Relatorio - INOVENTS.xlsx
+++ b/Integration-Quality/EMPRESAS/Relatorio - INOVENTS.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ5"/>
+  <dimension ref="A1:AQ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,35 +695,35 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>22746611</v>
+        <v>22780406</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>23542762</v>
+        <v>23572446</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>ACC01</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>45884.34997685185</v>
+        <v>45889.76509259259</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>45884.35454861111</v>
+        <v>45889.77414351852</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>5HQ3CX</t>
+          <t>IROQWB1</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -733,21 +733,21 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>SERVICO</t>
+          <t>LUCIANA MONTE</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Elaine Cristina Martins</t>
+          <t>Marcelo Soares de Azevedo</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Elaine Cristina Martins</t>
+          <t>Marcelo Soares de Azevedo</t>
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>45884.34930555556</v>
+        <v>45861.76458333333</v>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
@@ -766,32 +766,32 @@
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>Faturado</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>Serviço</t>
+          <t>Aéreo</t>
         </is>
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>Grupo Consolidacao</t>
+          <t>Grupo Vertex</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>Kontik Franstur Matriz/sao Paulo</t>
+          <t>Vertex Farmaceutica do Brasil</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -801,13 +801,11 @@
       </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>Sirena Textil</t>
-        </is>
-      </c>
-      <c r="Y2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Latam Airlines Brasil</t>
+        </is>
+      </c>
+      <c r="Y2" s="5" t="n">
+        <v>2971391236</v>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
@@ -815,19 +813,19 @@
         </is>
       </c>
       <c r="AA2" s="5" t="n">
-        <v>168578</v>
+        <v>169002</v>
       </c>
       <c r="AB2" s="5" t="n">
-        <v>5215.14</v>
+        <v>2610.64</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>0</v>
+        <v>91.56999999999999</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE2" s="5" t="n">
-        <v>0</v>
+        <v>261.06</v>
       </c>
       <c r="AF2" s="5" t="n">
         <v>0</v>
@@ -836,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>0</v>
+        <v>54.72</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
@@ -845,7 +843,7 @@
       </c>
       <c r="AJ2" s="5" t="inlineStr">
         <is>
-          <t>Necessário cadastrar um contrato para o cliente ""</t>
+          <t>Verificação de bilhetes: Bilhete 2971391236 já sendo utilizado para este fornecedor.</t>
         </is>
       </c>
       <c r="AK2" s="5" t="inlineStr">
@@ -855,17 +853,17 @@
       </c>
       <c r="AL2" s="5" t="inlineStr">
         <is>
-          <t>Contrato de fornecedor</t>
+          <t>Bilhete duplicado</t>
         </is>
       </c>
       <c r="AM2" s="5" t="inlineStr">
         <is>
-          <t>Análise Cadastro</t>
+          <t>Bilhete Já Contabilizado</t>
         </is>
       </c>
       <c r="AN2" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Duplicidade de Contabilização</t>
         </is>
       </c>
       <c r="AO2" s="5" t="inlineStr">
@@ -879,579 +877,6 @@
         </is>
       </c>
       <c r="AQ2" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="n">
-        <v>22741610</v>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>23538473</v>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>ACC01</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>45883.51908564815</v>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>45884.35450231482</v>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>5HTMEQ</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>SERVICO</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>Elaine Cristina Martins</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>Elaine Cristina Martins</t>
-        </is>
-      </c>
-      <c r="M3" s="6" t="n">
-        <v>45883.51875</v>
-      </c>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P3" s="5" t="inlineStr">
-        <is>
-          <t>OFF LINE</t>
-        </is>
-      </c>
-      <c r="Q3" s="5" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
-      <c r="R3" s="5" t="inlineStr">
-        <is>
-          <t>Faturado</t>
-        </is>
-      </c>
-      <c r="S3" s="5" t="inlineStr">
-        <is>
-          <t>Serviço</t>
-        </is>
-      </c>
-      <c r="T3" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="U3" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Consolidacao</t>
-        </is>
-      </c>
-      <c r="V3" s="5" t="inlineStr">
-        <is>
-          <t>Kontik Franstur Matriz/sao Paulo</t>
-        </is>
-      </c>
-      <c r="W3" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X3" s="5" t="inlineStr">
-        <is>
-          <t>Sirena Textil</t>
-        </is>
-      </c>
-      <c r="Y3" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z3" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-      <c r="AA3" s="5" t="n">
-        <v>168578</v>
-      </c>
-      <c r="AB3" s="5" t="n">
-        <v>5215.14</v>
-      </c>
-      <c r="AC3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI3" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ3" s="5" t="inlineStr">
-        <is>
-          <t>Necessário cadastrar um contrato para o cliente ""</t>
-        </is>
-      </c>
-      <c r="AK3" s="5" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="AL3" s="5" t="inlineStr">
-        <is>
-          <t>Contrato de fornecedor</t>
-        </is>
-      </c>
-      <c r="AM3" s="5" t="inlineStr">
-        <is>
-          <t>Análise Cadastro</t>
-        </is>
-      </c>
-      <c r="AN3" s="5" t="inlineStr">
-        <is>
-          <t>Dados do Fornecedor</t>
-        </is>
-      </c>
-      <c r="AO3" s="5" t="inlineStr">
-        <is>
-          <t>Qualidade dos dados</t>
-        </is>
-      </c>
-      <c r="AP3" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-      <c r="AQ3" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>22749021</v>
-      </c>
-      <c r="B4" s="5" t="n">
-        <v>23544966</v>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>ACC01</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>45884.61769675926</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>45884.61927083333</v>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">165858-414749-B </t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>EBOOKING</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> HOSPEDAGEM EM SANTA RITA DO SAPUCAÍ</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>Caio Jose Albuquerque Santos</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>Caio Jose Albuquerque Santos</t>
-        </is>
-      </c>
-      <c r="M4" s="6" t="n">
-        <v>45884.61736111111</v>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P4" s="5" t="inlineStr">
-        <is>
-          <t>OFF LINE</t>
-        </is>
-      </c>
-      <c r="Q4" s="5" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
-      <c r="R4" s="5" t="inlineStr">
-        <is>
-          <t>Faturado</t>
-        </is>
-      </c>
-      <c r="S4" s="5" t="inlineStr">
-        <is>
-          <t>Hotel</t>
-        </is>
-      </c>
-      <c r="T4" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="U4" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Claro Sa</t>
-        </is>
-      </c>
-      <c r="V4" s="5" t="inlineStr">
-        <is>
-          <t>Claro Sao Paulo (santo Amaro)</t>
-        </is>
-      </c>
-      <c r="W4" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X4" s="5" t="inlineStr">
-        <is>
-          <t>Hotel Amantykir</t>
-        </is>
-      </c>
-      <c r="Y4" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z4" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-      <c r="AA4" s="5" t="n">
-        <v>165858</v>
-      </c>
-      <c r="AB4" s="5" t="n">
-        <v>12852</v>
-      </c>
-      <c r="AC4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG4" s="5" t="n">
-        <v>642.6</v>
-      </c>
-      <c r="AH4" s="5" t="n">
-        <v>2053.6</v>
-      </c>
-      <c r="AI4" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> HOSPEDAGEM EM SANTA RITA DO SAPUCAÍ</t>
-        </is>
-      </c>
-      <c r="AJ4" s="5" t="inlineStr">
-        <is>
-          <t>Centro de custo não preenchido! (ACC01)</t>
-        </is>
-      </c>
-      <c r="AK4" s="5" t="inlineStr">
-        <is>
-          <t>EBOOKING</t>
-        </is>
-      </c>
-      <c r="AL4" s="5" t="inlineStr">
-        <is>
-          <t>Centro de custo</t>
-        </is>
-      </c>
-      <c r="AM4" s="5" t="inlineStr">
-        <is>
-          <t>Falta de informação Gerencial</t>
-        </is>
-      </c>
-      <c r="AN4" s="5" t="inlineStr">
-        <is>
-          <t>Dados do Fornecedor</t>
-        </is>
-      </c>
-      <c r="AO4" s="5" t="inlineStr">
-        <is>
-          <t>Qualidade dos dados</t>
-        </is>
-      </c>
-      <c r="AP4" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-      <c r="AQ4" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>22749395</v>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>23545373</v>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>ACC01</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>45884.66975694444</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>45884.67158564815</v>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>03 a 05 dias</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>5H2OKX</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>SERVICO</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Elaine Cristina Martins</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>Elaine Cristina Martins</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>45884.66944444444</v>
-      </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P5" s="5" t="inlineStr">
-        <is>
-          <t>OFF LINE</t>
-        </is>
-      </c>
-      <c r="Q5" s="5" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
-      <c r="R5" s="5" t="inlineStr">
-        <is>
-          <t>Faturado</t>
-        </is>
-      </c>
-      <c r="S5" s="5" t="inlineStr">
-        <is>
-          <t>Serviço</t>
-        </is>
-      </c>
-      <c r="T5" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="U5" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Consolidacao</t>
-        </is>
-      </c>
-      <c r="V5" s="5" t="inlineStr">
-        <is>
-          <t>Kontik Franstur Matriz/sao Paulo</t>
-        </is>
-      </c>
-      <c r="W5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X5" s="5" t="inlineStr">
-        <is>
-          <t>Sirena Textil</t>
-        </is>
-      </c>
-      <c r="Y5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z5" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-      <c r="AA5" s="5" t="n">
-        <v>168578</v>
-      </c>
-      <c r="AB5" s="5" t="n">
-        <v>5215.14</v>
-      </c>
-      <c r="AC5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ5" s="5" t="inlineStr">
-        <is>
-          <t>Necessário informar a filial do cliente "Kontik Franstur Matriz/sao Paulo" em seu contrato</t>
-        </is>
-      </c>
-      <c r="AK5" s="5" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="AL5" s="5" t="inlineStr">
-        <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="AM5" s="5" t="inlineStr">
-        <is>
-          <t>Análise Benner</t>
-        </is>
-      </c>
-      <c r="AN5" s="5" t="inlineStr">
-        <is>
-          <t>Sistema</t>
-        </is>
-      </c>
-      <c r="AO5" s="5" t="inlineStr">
-        <is>
-          <t>Qualidade dos dados</t>
-        </is>
-      </c>
-      <c r="AP5" s="5" t="inlineStr">
-        <is>
-          <t>INOVENTS</t>
-        </is>
-      </c>
-      <c r="AQ5" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>

</xml_diff>

<commit_message>
Remove outdated PDF reports and Excel files from Integration-Quality directory; update Processado Erro.xlsx with new data.
</commit_message>
<xml_diff>
--- a/Integration-Quality/EMPRESAS/Relatorio - INOVENTS.xlsx
+++ b/Integration-Quality/EMPRESAS/Relatorio - INOVENTS.xlsx
@@ -695,10 +695,10 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>24599611</v>
+        <v>24802417</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>25425647</v>
+        <v>25643620</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
@@ -706,108 +706,106 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>46157.57175925926</v>
+        <v>46196.37805555556</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>46157.57332175926</v>
+        <v>46196.55409722222</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>03 a 05 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">191854-503382-A </t>
+          <t>GRISFY</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>EBOOKING</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ana Clara Rodrigues </t>
+          <t>JARDELINO PEREIRA DA COSTA</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>INEZ LOPES RIBEIRO DOS SANTOS TELES</t>
+          <t>Flavio Alexandre Ribeiro de Mello Mazzola</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>INEZ LOPES RIBEIRO DOS SANTOS TELES</t>
+          <t>Flavio Alexandre Ribeiro de Mello Mazzola</t>
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>46157.57152777778</v>
+        <v>46189</v>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
+          <t>CLOVIS MORO</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>Cartão de crédito</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Enesa</t>
+        </is>
+      </c>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
+          <t>Enesa Engenharia</t>
+        </is>
+      </c>
+      <c r="W2" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
-        <is>
-          <t>OFF LINE</t>
-        </is>
-      </c>
-      <c r="Q2" s="5" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
-      <c r="R2" s="5" t="inlineStr">
-        <is>
-          <t>Faturado</t>
-        </is>
-      </c>
-      <c r="S2" s="5" t="inlineStr">
-        <is>
-          <t>Serviço</t>
-        </is>
-      </c>
-      <c r="T2" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="U2" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Syngenta</t>
-        </is>
-      </c>
-      <c r="V2" s="5" t="inlineStr">
-        <is>
-          <t>Syngenta Crop</t>
-        </is>
-      </c>
-      <c r="W2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>Fabio Roberto Lima Lais</t>
-        </is>
-      </c>
-      <c r="Y2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Latam Airlines Brasil</t>
+        </is>
+      </c>
+      <c r="Y2" s="5" t="n">
+        <v>2292010132</v>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
@@ -815,13 +813,13 @@
         </is>
       </c>
       <c r="AA2" s="5" t="n">
-        <v>191854</v>
+        <v>201745</v>
       </c>
       <c r="AB2" s="5" t="n">
-        <v>4000</v>
+        <v>2480</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>0</v>
+        <v>92.84</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
@@ -836,31 +834,31 @@
         <v>0</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>330.45</v>
+        <v>0</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 TURMA- SEEDCARE </t>
+          <t>Reserva importada via planilha. Solicitação: |PC:</t>
         </is>
       </c>
       <c r="AJ2" s="5" t="inlineStr">
         <is>
-          <t>Matrícula não preenchida! (ACC01)</t>
+          <t xml:space="preserve"> Módulo Operações    -&gt; Configurações      -&gt; Configurações do sistema turismo        -&gt; Importação das vendas          -&gt; Entradas/Saídas  Para o </t>
         </is>
       </c>
       <c r="AK2" s="5" t="inlineStr">
         <is>
-          <t>EBOOKING</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="AL2" s="5" t="inlineStr">
         <is>
-          <t>Matrícula</t>
+          <t>Pagamento não permitido para cobrança</t>
         </is>
       </c>
       <c r="AM2" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Forma PG. e REC.</t>
         </is>
       </c>
       <c r="AN2" s="5" t="inlineStr">
@@ -886,63 +884,63 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>10927909</v>
+        <v>24802417</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>12272973</v>
+        <v>25643621</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>ACC01</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>43383.66349537037</v>
+        <v>46196.37805555556</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>46154.42668981481</v>
+        <v>46196.55409722222</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>31 dias ou +</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>HHWJMP</t>
+          <t>GRISFY</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>EBOOKING</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>VASCONCELOS JUNIOR/JOSE</t>
+          <t>JORGE DA COSTA SILVA</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Ana Carolina de Carvalho Svartman</t>
+          <t>Flavio Alexandre Ribeiro de Mello Mazzola</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Ana Carolina de Carvalho Svartman</t>
+          <t>Flavio Alexandre Ribeiro de Mello Mazzola</t>
         </is>
       </c>
       <c r="M3" s="6" t="n">
-        <v>43384.38821759259</v>
+        <v>46189</v>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>CLOVIS MORO</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
@@ -957,14 +955,14 @@
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
           <t>Cartão de crédito</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
-        <is>
-          <t>Cartão de crédito</t>
-        </is>
-      </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
           <t>Aéreo</t>
@@ -977,42 +975,40 @@
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>Grupo Diageo</t>
+          <t>Grupo Enesa</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>Ypioca Industrial de Bebidas S a</t>
+          <t>Enesa Engenharia</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
         <is>
-          <t>Cliente FEE no POS</t>
+          <t>-</t>
         </is>
       </c>
       <c r="X3" s="5" t="inlineStr">
         <is>
-          <t>Gol Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>4311970720</v>
+        <v>2292010133</v>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
           <t>INOVENTS</t>
         </is>
       </c>
-      <c r="AA3" s="5" t="inlineStr">
-        <is>
-          <t>EV17608</t>
-        </is>
+      <c r="AA3" s="5" t="n">
+        <v>201745</v>
       </c>
       <c r="AB3" s="5" t="n">
-        <v>658.42</v>
+        <v>2480</v>
       </c>
       <c r="AC3" s="5" t="n">
-        <v>30.94</v>
+        <v>92.84</v>
       </c>
       <c r="AD3" s="5" t="n">
         <v>0</v>
@@ -1021,37 +1017,37 @@
         <v>0</v>
       </c>
       <c r="AF3" s="5" t="n">
-        <v>30.94</v>
+        <v>0</v>
       </c>
       <c r="AG3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AH3" s="5" t="n">
-        <v>48.26</v>
+        <v>0</v>
       </c>
       <c r="AI3" s="5" t="inlineStr">
         <is>
-          <t>PNR gerado via WebService NSGOL (172.16.1.194)</t>
+          <t>Reserva importada via planilha. Solicitação: |PC:</t>
         </is>
       </c>
       <c r="AJ3" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo não preenchido! (ACC01)</t>
+          <t xml:space="preserve"> Módulo Operações    -&gt; Configurações      -&gt; Configurações do sistema turismo        -&gt; Importação das vendas          -&gt; Entradas/Saídas  Para o </t>
         </is>
       </c>
       <c r="AK3" s="5" t="inlineStr">
         <is>
-          <t>EBOOKING</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="AL3" s="5" t="inlineStr">
         <is>
-          <t>Centro de custo</t>
+          <t>Pagamento não permitido para cobrança</t>
         </is>
       </c>
       <c r="AM3" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Forma PG. e REC.</t>
         </is>
       </c>
       <c r="AN3" s="5" t="inlineStr">

</xml_diff>